<commit_message>
feat(orcamento): lanca equipe de TI mai-jul/26
Vinicius dividido em salario bruto + encargos, mesmo tratamento da
Geovanna. Aumento permanente de R$ 500 a partir de 05/08 (bruto de
R$ 2.570,52 para R$ 3.070,52) refletido no planejado de ago a dez;
orcamento total sobe para R$ 398.352,68.

Desvios do periodo (acumulado mai-jul):
- Jonathan R$ 6.300/mes contra R$ 10.000 orcados: -R$ 11.100, o maior
  desvio em reais de todo o orcamento
- Elias zerado nos tres meses: -R$ 3.195

Ambos registrados na aba Pendencias — se forem o novo padrao, o
planejado de ago a dez precisa ser revisado para baixo.

Registrada tambem a observacao de que o orcado de custo total do
Vinicius implica encargos de 111% sobre o bruto, acima do usual.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -17,8 +17,8 @@
     <sheet name="Como usar" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparativo'!$A$5:$N$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Planejado'!$A$4:$P$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparativo'!$A$5:$N$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Planejado'!$A$4:$P$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1121,15 +1121,15 @@
         </is>
       </c>
       <c r="C6" s="8">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$B$5:$B$26,"Jurídico",Planejado!$C$5:$C$26,"Equipe")</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$B$5:$B$27,"Jurídico",Planejado!$C$5:$C$27,"Equipe")</f>
         <v/>
       </c>
       <c r="D6" s="8">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$B$6:$B$27,"Jurídico",Comparativo!$C$6:$C$27,"Equipe")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$B$6:$B$28,"Jurídico",Comparativo!$C$6:$C$28,"Equipe")</f>
         <v/>
       </c>
       <c r="E6" s="8">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$B$6:$B$27,"Jurídico",Comparativo!$C$6:$C$27,"Equipe")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$B$6:$B$28,"Jurídico",Comparativo!$C$6:$C$28,"Equipe")</f>
         <v/>
       </c>
       <c r="F6" s="8">
@@ -1145,7 +1145,7 @@
         <v/>
       </c>
       <c r="I6" s="10">
-        <f>COUNTIFS(Comparativo!$P$6:$P$27,"&gt;0",Comparativo!$B$6:$B$27,"Jurídico",Comparativo!$C$6:$C$27,"Equipe")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$27,"?*",Comparativo!$B$6:$B$27,"Jurídico",Comparativo!$C$6:$C$27,"Equipe")</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$28,"&gt;0",Comparativo!$B$6:$B$28,"Jurídico",Comparativo!$C$6:$C$28,"Equipe")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$28,"?*",Comparativo!$B$6:$B$28,"Jurídico",Comparativo!$C$6:$C$28,"Equipe")</f>
         <v/>
       </c>
     </row>
@@ -1161,15 +1161,15 @@
         </is>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$B$5:$B$26,"Jurídico",Planejado!$C$5:$C$26,"Despesas")</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$B$5:$B$27,"Jurídico",Planejado!$C$5:$C$27,"Despesas")</f>
         <v/>
       </c>
       <c r="D7" s="8">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$B$6:$B$27,"Jurídico",Comparativo!$C$6:$C$27,"Despesas")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$B$6:$B$28,"Jurídico",Comparativo!$C$6:$C$28,"Despesas")</f>
         <v/>
       </c>
       <c r="E7" s="8">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$B$6:$B$27,"Jurídico",Comparativo!$C$6:$C$27,"Despesas")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$B$6:$B$28,"Jurídico",Comparativo!$C$6:$C$28,"Despesas")</f>
         <v/>
       </c>
       <c r="F7" s="8">
@@ -1185,7 +1185,7 @@
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>COUNTIFS(Comparativo!$P$6:$P$27,"&gt;0",Comparativo!$B$6:$B$27,"Jurídico",Comparativo!$C$6:$C$27,"Despesas")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$27,"?*",Comparativo!$B$6:$B$27,"Jurídico",Comparativo!$C$6:$C$27,"Despesas")</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$28,"&gt;0",Comparativo!$B$6:$B$28,"Jurídico",Comparativo!$C$6:$C$28,"Despesas")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$28,"?*",Comparativo!$B$6:$B$28,"Jurídico",Comparativo!$C$6:$C$28,"Despesas")</f>
         <v/>
       </c>
     </row>
@@ -1201,15 +1201,15 @@
         </is>
       </c>
       <c r="C8" s="12">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="F8" s="12">
@@ -1225,7 +1225,7 @@
         <v/>
       </c>
       <c r="I8" s="14">
-        <f>COUNTIFS(Comparativo!$P$6:$P$27,"&gt;0",Comparativo!$B$6:$B$27,"Jurídico")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$27,"?*",Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$28,"&gt;0",Comparativo!$B$6:$B$28,"Jurídico")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$28,"?*",Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
     </row>
@@ -1241,15 +1241,15 @@
         </is>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$B$5:$B$26,"TI",Planejado!$C$5:$C$26,"Equipe")</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$B$5:$B$27,"TI",Planejado!$C$5:$C$27,"Equipe")</f>
         <v/>
       </c>
       <c r="D9" s="8">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$B$6:$B$27,"TI",Comparativo!$C$6:$C$27,"Equipe")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$B$6:$B$28,"TI",Comparativo!$C$6:$C$28,"Equipe")</f>
         <v/>
       </c>
       <c r="E9" s="8">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$B$6:$B$27,"TI",Comparativo!$C$6:$C$27,"Equipe")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$B$6:$B$28,"TI",Comparativo!$C$6:$C$28,"Equipe")</f>
         <v/>
       </c>
       <c r="F9" s="8">
@@ -1265,7 +1265,7 @@
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>COUNTIFS(Comparativo!$P$6:$P$27,"&gt;0",Comparativo!$B$6:$B$27,"TI",Comparativo!$C$6:$C$27,"Equipe")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$27,"?*",Comparativo!$B$6:$B$27,"TI",Comparativo!$C$6:$C$27,"Equipe")</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$28,"&gt;0",Comparativo!$B$6:$B$28,"TI",Comparativo!$C$6:$C$28,"Equipe")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$28,"?*",Comparativo!$B$6:$B$28,"TI",Comparativo!$C$6:$C$28,"Equipe")</f>
         <v/>
       </c>
     </row>
@@ -1281,15 +1281,15 @@
         </is>
       </c>
       <c r="C10" s="8">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$B$5:$B$26,"TI",Planejado!$C$5:$C$26,"Despesas")</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$B$5:$B$27,"TI",Planejado!$C$5:$C$27,"Despesas")</f>
         <v/>
       </c>
       <c r="D10" s="8">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$B$6:$B$27,"TI",Comparativo!$C$6:$C$27,"Despesas")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$B$6:$B$28,"TI",Comparativo!$C$6:$C$28,"Despesas")</f>
         <v/>
       </c>
       <c r="E10" s="8">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$B$6:$B$27,"TI",Comparativo!$C$6:$C$27,"Despesas")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$B$6:$B$28,"TI",Comparativo!$C$6:$C$28,"Despesas")</f>
         <v/>
       </c>
       <c r="F10" s="8">
@@ -1305,7 +1305,7 @@
         <v/>
       </c>
       <c r="I10" s="10">
-        <f>COUNTIFS(Comparativo!$P$6:$P$27,"&gt;0",Comparativo!$B$6:$B$27,"TI",Comparativo!$C$6:$C$27,"Despesas")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$27,"?*",Comparativo!$B$6:$B$27,"TI",Comparativo!$C$6:$C$27,"Despesas")</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$28,"&gt;0",Comparativo!$B$6:$B$28,"TI",Comparativo!$C$6:$C$28,"Despesas")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$28,"?*",Comparativo!$B$6:$B$28,"TI",Comparativo!$C$6:$C$28,"Despesas")</f>
         <v/>
       </c>
     </row>
@@ -1321,15 +1321,15 @@
         </is>
       </c>
       <c r="C11" s="12">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="F11" s="12">
@@ -1345,7 +1345,7 @@
         <v/>
       </c>
       <c r="I11" s="14">
-        <f>COUNTIFS(Comparativo!$P$6:$P$27,"&gt;0",Comparativo!$B$6:$B$27,"TI")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$27,"?*",Comparativo!$B$6:$B$27,"TI")</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$28,"&gt;0",Comparativo!$B$6:$B$28,"TI")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$28,"?*",Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
     </row>
@@ -1357,15 +1357,15 @@
       </c>
       <c r="B12" s="15" t="inlineStr"/>
       <c r="C12" s="16">
-        <f>SUM(Planejado!$P$5:$P$26)</f>
+        <f>SUM(Planejado!$P$5:$P$27)</f>
         <v/>
       </c>
       <c r="D12" s="16">
-        <f>SUM(Comparativo!$I$6:$I$27)</f>
+        <f>SUM(Comparativo!$I$6:$I$28)</f>
         <v/>
       </c>
       <c r="E12" s="16">
-        <f>SUM(Comparativo!$J$6:$J$27)</f>
+        <f>SUM(Comparativo!$J$6:$J$28)</f>
         <v/>
       </c>
       <c r="F12" s="16">
@@ -1381,7 +1381,7 @@
         <v/>
       </c>
       <c r="I12" s="18">
-        <f>COUNTIFS(Comparativo!$P$6:$P$27,"&gt;0")&amp;" de "&amp;COUNTA(Comparativo!$A$6:$A$27)</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$28,"&gt;0")&amp;" de "&amp;COUNTA(Comparativo!$A$6:$A$28)</f>
         <v/>
       </c>
     </row>
@@ -1435,23 +1435,23 @@
         <v>1</v>
       </c>
       <c r="B17" s="21">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A17),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A17),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="C17" s="21">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A17),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A17),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="D17" s="22">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A17),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A17),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="E17" s="22">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A17),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A17),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="F17" s="22">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A17),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A17),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="G17" s="23">
@@ -1464,23 +1464,23 @@
         <v>2</v>
       </c>
       <c r="B18" s="21">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A18),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A18),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A18),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A18),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="D18" s="22">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A18),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A18),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A18),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A18),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A18),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A18),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="G18" s="23">
@@ -1493,23 +1493,23 @@
         <v>3</v>
       </c>
       <c r="B19" s="21">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A19),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A19),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="C19" s="21">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A19),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A19),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="D19" s="22">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A19),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A19),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="E19" s="22">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A19),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A19),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="F19" s="22">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A19),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A19),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="G19" s="23">
@@ -1522,23 +1522,23 @@
         <v>4</v>
       </c>
       <c r="B20" s="21">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A20),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A20),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A20),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A20),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="D20" s="22">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A20),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A20),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A20),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A20),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A20),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A20),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="G20" s="23">
@@ -1551,23 +1551,23 @@
         <v>5</v>
       </c>
       <c r="B21" s="21">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A21),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A21),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="C21" s="21">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A21),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A21),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="D21" s="22">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A21),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A21),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="E21" s="22">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A21),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A21),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="F21" s="22">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$27,MATCH(LARGE(Comparativo!$O$6:$O$27,A21),Comparativo!$O$6:$O$27,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$28,MATCH(LARGE(Comparativo!$O$6:$O$28,A21),Comparativo!$O$6:$O$28,0)),"")</f>
         <v/>
       </c>
       <c r="G21" s="23">
@@ -1591,7 +1591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3181,57 +3181,123 @@
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="34">
+        <f>Planejado!A27</f>
+        <v/>
+      </c>
+      <c r="B28" s="34">
+        <f>Planejado!B27</f>
+        <v/>
+      </c>
+      <c r="C28" s="34">
+        <f>Planejado!C27</f>
+        <v/>
+      </c>
+      <c r="D28" s="35">
+        <f>Planejado!D27</f>
+        <v/>
+      </c>
+      <c r="E28" s="34">
+        <f>Planejado!G27</f>
+        <v/>
+      </c>
+      <c r="F28" s="36">
+        <f>INDEX(Planejado!$H27:$O27,$D$3)</f>
+        <v/>
+      </c>
+      <c r="G28" s="36">
+        <f>INDEX(Realizado!$H27:$O27,$D$3)</f>
+        <v/>
+      </c>
+      <c r="H28" s="36">
+        <f>G28-F28</f>
+        <v/>
+      </c>
+      <c r="I28" s="36">
+        <f>SUMPRODUCT((COLUMN(Planejado!$H$4:$O$4)-COLUMN(Planejado!$H$4)+1&lt;=$D$3)*Planejado!$H27:$O27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="36">
+        <f>SUMPRODUCT((COLUMN(Realizado!$H$4:$O$4)-COLUMN(Realizado!$H$4)+1&lt;=$D$3)*Realizado!$H27:$O27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="36">
+        <f>J28-I28</f>
+        <v/>
+      </c>
+      <c r="L28" s="37">
+        <f>IFERROR(K28/I28,"")</f>
+        <v/>
+      </c>
+      <c r="M28" s="37">
+        <f>IFERROR(J28/I28,"")</f>
+        <v/>
+      </c>
+      <c r="N28" s="38">
+        <f>IF(P28=0,"Sem lançamento",IF(AND(I28=0,J28=0),"—",IF(I28=0,"Não orçado",IF(K28&gt;0.05*I28,"Acima do orçado",IF(K28&lt;-0.05*I28,"Abaixo do orçado","Dentro do orçado")))))</f>
+        <v/>
+      </c>
+      <c r="O28" s="27">
+        <f>IF(K28&gt;1,K28+ROW()/1000000,"")</f>
+        <v/>
+      </c>
+      <c r="P28" s="39">
+        <f>SUMPRODUCT((COLUMN(Realizado!$H$4:$O$4)-COLUMN(Realizado!$H$4)+1&lt;=$D$3)*(Realizado!$H27:$O27&lt;&gt;""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B28" s="15" t="n"/>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
-      <c r="E28" s="15" t="n"/>
-      <c r="F28" s="16">
-        <f>SUM(F6:F27)</f>
-        <v/>
-      </c>
-      <c r="G28" s="16">
-        <f>SUM(G6:G27)</f>
-        <v/>
-      </c>
-      <c r="H28" s="16">
-        <f>SUM(H6:H27)</f>
-        <v/>
-      </c>
-      <c r="I28" s="16">
-        <f>SUM(I6:I27)</f>
-        <v/>
-      </c>
-      <c r="J28" s="16">
-        <f>SUM(J6:J27)</f>
-        <v/>
-      </c>
-      <c r="K28" s="16">
-        <f>SUM(K6:K27)</f>
-        <v/>
-      </c>
-      <c r="L28" s="40">
-        <f>IFERROR(K28/I28,"")</f>
-        <v/>
-      </c>
-      <c r="M28" s="40">
-        <f>IFERROR(J28/I28,"")</f>
-        <v/>
-      </c>
-      <c r="N28" s="15" t="n"/>
+      <c r="B29" s="15" t="n"/>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="16">
+        <f>SUM(F6:F28)</f>
+        <v/>
+      </c>
+      <c r="G29" s="16">
+        <f>SUM(G6:G28)</f>
+        <v/>
+      </c>
+      <c r="H29" s="16">
+        <f>SUM(H6:H28)</f>
+        <v/>
+      </c>
+      <c r="I29" s="16">
+        <f>SUM(I6:I28)</f>
+        <v/>
+      </c>
+      <c r="J29" s="16">
+        <f>SUM(J6:J28)</f>
+        <v/>
+      </c>
+      <c r="K29" s="16">
+        <f>SUM(K6:K28)</f>
+        <v/>
+      </c>
+      <c r="L29" s="40">
+        <f>IFERROR(K29/I29,"")</f>
+        <v/>
+      </c>
+      <c r="M29" s="40">
+        <f>IFERROR(J29/I29,"")</f>
+        <v/>
+      </c>
+      <c r="N29" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:N27"/>
+  <autoFilter ref="A5:N28"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H6:H27">
+  <conditionalFormatting sqref="H6:H28">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3239,7 +3305,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K27">
+  <conditionalFormatting sqref="K6:K28">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3262,7 +3328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4011,12 +4077,12 @@
       </c>
       <c r="D15" s="35" t="inlineStr">
         <is>
-          <t>Vinicius Di Franco</t>
+          <t>Vinicius Di Franco — salário bruto</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Analista Administrativo</t>
+          <t>Analista Administrativo — aumento de R$ 2.570,52 para R$ 3.070,52 a partir de 05/08/26</t>
         </is>
       </c>
       <c r="F15" s="34" t="inlineStr">
@@ -4030,28 +4096,28 @@
         </is>
       </c>
       <c r="H15" s="36" t="n">
-        <v>5416.525</v>
+        <v>2570.52</v>
       </c>
       <c r="I15" s="36" t="n">
-        <v>5416.525</v>
+        <v>2570.52</v>
       </c>
       <c r="J15" s="36" t="n">
-        <v>5416.525</v>
+        <v>2570.52</v>
       </c>
       <c r="K15" s="36" t="n">
-        <v>5416.525</v>
+        <v>3070.52</v>
       </c>
       <c r="L15" s="36" t="n">
-        <v>5416.525</v>
+        <v>3070.52</v>
       </c>
       <c r="M15" s="36" t="n">
-        <v>5416.525</v>
+        <v>3070.52</v>
       </c>
       <c r="N15" s="36" t="n">
-        <v>5416.525</v>
+        <v>3070.52</v>
       </c>
       <c r="O15" s="36" t="n">
-        <v>5416.525</v>
+        <v>3070.52</v>
       </c>
       <c r="P15" s="41">
         <f>SUM(H15:O15)</f>
@@ -4061,7 +4127,7 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="34" t="inlineStr">
         <is>
-          <t>TI-E02</t>
+          <t>TI-E01B</t>
         </is>
       </c>
       <c r="B16" s="34" t="inlineStr">
@@ -4076,47 +4142,47 @@
       </c>
       <c r="D16" s="35" t="inlineStr">
         <is>
-          <t>Elias Benedito</t>
+          <t>Vinicius Di Franco — encargos e benefícios</t>
         </is>
       </c>
       <c r="E16" s="35" t="inlineStr">
         <is>
-          <t>Suporte Técnico Terceirizado</t>
+          <t>INSS patronal, FGTS, provisões de 13º e férias, benefícios — PREENCHER</t>
         </is>
       </c>
       <c r="F16" s="34" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="G16" s="34" t="inlineStr">
         <is>
-          <t>Pessoal - PJ</t>
+          <t>Encargos e Benefícios - CLT</t>
         </is>
       </c>
       <c r="H16" s="36" t="n">
-        <v>1065</v>
+        <v>2846.005</v>
       </c>
       <c r="I16" s="36" t="n">
-        <v>1065</v>
+        <v>2846.005</v>
       </c>
       <c r="J16" s="36" t="n">
-        <v>1065</v>
+        <v>2846.005</v>
       </c>
       <c r="K16" s="36" t="n">
-        <v>1065</v>
+        <v>2846.005</v>
       </c>
       <c r="L16" s="36" t="n">
-        <v>1065</v>
+        <v>2846.005</v>
       </c>
       <c r="M16" s="36" t="n">
-        <v>1065</v>
+        <v>2846.005</v>
       </c>
       <c r="N16" s="36" t="n">
-        <v>1065</v>
+        <v>2846.005</v>
       </c>
       <c r="O16" s="36" t="n">
-        <v>1065</v>
+        <v>2846.005</v>
       </c>
       <c r="P16" s="41">
         <f>SUM(H16:O16)</f>
@@ -4126,7 +4192,7 @@
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="34" t="inlineStr">
         <is>
-          <t>TI-E03</t>
+          <t>TI-E02</t>
         </is>
       </c>
       <c r="B17" s="34" t="inlineStr">
@@ -4141,12 +4207,12 @@
       </c>
       <c r="D17" s="35" t="inlineStr">
         <is>
-          <t>Jonathan</t>
+          <t>Elias Benedito</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Consultor</t>
+          <t>Suporte Técnico Terceirizado</t>
         </is>
       </c>
       <c r="F17" s="34" t="inlineStr">
@@ -4160,28 +4226,28 @@
         </is>
       </c>
       <c r="H17" s="36" t="n">
-        <v>10000</v>
+        <v>1065</v>
       </c>
       <c r="I17" s="36" t="n">
-        <v>10000</v>
+        <v>1065</v>
       </c>
       <c r="J17" s="36" t="n">
-        <v>10000</v>
+        <v>1065</v>
       </c>
       <c r="K17" s="36" t="n">
-        <v>10000</v>
+        <v>1065</v>
       </c>
       <c r="L17" s="36" t="n">
-        <v>10000</v>
+        <v>1065</v>
       </c>
       <c r="M17" s="36" t="n">
-        <v>10000</v>
+        <v>1065</v>
       </c>
       <c r="N17" s="36" t="n">
-        <v>10000</v>
+        <v>1065</v>
       </c>
       <c r="O17" s="36" t="n">
-        <v>10000</v>
+        <v>1065</v>
       </c>
       <c r="P17" s="41">
         <f>SUM(H17:O17)</f>
@@ -4191,7 +4257,7 @@
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="34" t="inlineStr">
         <is>
-          <t>TI-D01</t>
+          <t>TI-E03</t>
         </is>
       </c>
       <c r="B18" s="34" t="inlineStr">
@@ -4201,48 +4267,52 @@
       </c>
       <c r="C18" s="34" t="inlineStr">
         <is>
-          <t>Despesas</t>
+          <t>Equipe</t>
         </is>
       </c>
       <c r="D18" s="35" t="inlineStr">
         <is>
-          <t>Peças de Manutenção</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="E18" s="35" t="inlineStr">
         <is>
-          <t>Tela, teclado, carcaça, mouses de reposição, carregadores etc.</t>
-        </is>
-      </c>
-      <c r="F18" s="34" t="inlineStr"/>
+          <t>Consultor</t>
+        </is>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="G18" s="34" t="inlineStr">
         <is>
-          <t>Equipamentos Eletrônicos Diversos</t>
+          <t>Pessoal - PJ</t>
         </is>
       </c>
       <c r="H18" s="36" t="n">
-        <v>810</v>
+        <v>10000</v>
       </c>
       <c r="I18" s="36" t="n">
-        <v>810</v>
+        <v>10000</v>
       </c>
       <c r="J18" s="36" t="n">
-        <v>810</v>
+        <v>10000</v>
       </c>
       <c r="K18" s="36" t="n">
-        <v>810</v>
+        <v>10000</v>
       </c>
       <c r="L18" s="36" t="n">
-        <v>810</v>
+        <v>10000</v>
       </c>
       <c r="M18" s="36" t="n">
-        <v>810</v>
+        <v>10000</v>
       </c>
       <c r="N18" s="36" t="n">
-        <v>810</v>
+        <v>10000</v>
       </c>
       <c r="O18" s="36" t="n">
-        <v>810</v>
+        <v>10000</v>
       </c>
       <c r="P18" s="41">
         <f>SUM(H18:O18)</f>
@@ -4252,7 +4322,7 @@
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="34" t="inlineStr">
         <is>
-          <t>TI-D02</t>
+          <t>TI-D01</t>
         </is>
       </c>
       <c r="B19" s="34" t="inlineStr">
@@ -4267,43 +4337,43 @@
       </c>
       <c r="D19" s="35" t="inlineStr">
         <is>
-          <t>Backup em Nuvem</t>
+          <t>Peças de Manutenção</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Serviço de backup em nuvem para servidor — RATEIO A DEFINIR</t>
+          <t>Tela, teclado, carcaça, mouses de reposição, carregadores etc.</t>
         </is>
       </c>
       <c r="F19" s="34" t="inlineStr"/>
       <c r="G19" s="34" t="inlineStr">
         <is>
-          <t>Licenças de Softwares</t>
+          <t>Equipamentos Eletrônicos Diversos</t>
         </is>
       </c>
       <c r="H19" s="36" t="n">
-        <v>825</v>
+        <v>810</v>
       </c>
       <c r="I19" s="36" t="n">
-        <v>825</v>
+        <v>810</v>
       </c>
       <c r="J19" s="36" t="n">
-        <v>825</v>
+        <v>810</v>
       </c>
       <c r="K19" s="36" t="n">
-        <v>825</v>
+        <v>810</v>
       </c>
       <c r="L19" s="36" t="n">
-        <v>825</v>
+        <v>810</v>
       </c>
       <c r="M19" s="36" t="n">
-        <v>825</v>
+        <v>810</v>
       </c>
       <c r="N19" s="36" t="n">
-        <v>825</v>
+        <v>810</v>
       </c>
       <c r="O19" s="36" t="n">
-        <v>825</v>
+        <v>810</v>
       </c>
       <c r="P19" s="41">
         <f>SUM(H19:O19)</f>
@@ -4313,7 +4383,7 @@
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="34" t="inlineStr">
         <is>
-          <t>TI-D03</t>
+          <t>TI-D02</t>
         </is>
       </c>
       <c r="B20" s="34" t="inlineStr">
@@ -4328,12 +4398,12 @@
       </c>
       <c r="D20" s="35" t="inlineStr">
         <is>
-          <t>Inteligência Artificial (Adapta)</t>
+          <t>Backup em Nuvem</t>
         </is>
       </c>
       <c r="E20" s="35" t="inlineStr">
         <is>
-          <t>Plataforma de IA para utilização de agentes — RATEIO A DEFINIR</t>
+          <t>Serviço de backup em nuvem para servidor — RATEIO A DEFINIR</t>
         </is>
       </c>
       <c r="F20" s="34" t="inlineStr"/>
@@ -4343,28 +4413,28 @@
         </is>
       </c>
       <c r="H20" s="36" t="n">
-        <v>1300</v>
+        <v>825</v>
       </c>
       <c r="I20" s="36" t="n">
-        <v>1300</v>
+        <v>825</v>
       </c>
       <c r="J20" s="36" t="n">
-        <v>1600</v>
+        <v>825</v>
       </c>
       <c r="K20" s="36" t="n">
-        <v>1600</v>
+        <v>825</v>
       </c>
       <c r="L20" s="36" t="n">
-        <v>1600</v>
+        <v>825</v>
       </c>
       <c r="M20" s="36" t="n">
-        <v>1600</v>
+        <v>825</v>
       </c>
       <c r="N20" s="36" t="n">
-        <v>1600</v>
+        <v>825</v>
       </c>
       <c r="O20" s="36" t="n">
-        <v>1600</v>
+        <v>825</v>
       </c>
       <c r="P20" s="41">
         <f>SUM(H20:O20)</f>
@@ -4374,7 +4444,7 @@
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="34" t="inlineStr">
         <is>
-          <t>TI-D04</t>
+          <t>TI-D03</t>
         </is>
       </c>
       <c r="B21" s="34" t="inlineStr">
@@ -4389,12 +4459,12 @@
       </c>
       <c r="D21" s="35" t="inlineStr">
         <is>
-          <t>Antivírus</t>
+          <t>Inteligência Artificial (Adapta)</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Proteção para equipamentos — RATEIO A DEFINIR</t>
+          <t>Plataforma de IA para utilização de agentes — RATEIO A DEFINIR</t>
         </is>
       </c>
       <c r="F21" s="34" t="inlineStr"/>
@@ -4404,28 +4474,28 @@
         </is>
       </c>
       <c r="H21" s="36" t="n">
-        <v>240</v>
+        <v>1300</v>
       </c>
       <c r="I21" s="36" t="n">
-        <v>240</v>
+        <v>1300</v>
       </c>
       <c r="J21" s="36" t="n">
-        <v>240</v>
+        <v>1600</v>
       </c>
       <c r="K21" s="36" t="n">
-        <v>240</v>
+        <v>1600</v>
       </c>
       <c r="L21" s="36" t="n">
-        <v>240</v>
+        <v>1600</v>
       </c>
       <c r="M21" s="36" t="n">
-        <v>240</v>
+        <v>1600</v>
       </c>
       <c r="N21" s="36" t="n">
-        <v>240</v>
+        <v>1600</v>
       </c>
       <c r="O21" s="36" t="n">
-        <v>240</v>
+        <v>1600</v>
       </c>
       <c r="P21" s="41">
         <f>SUM(H21:O21)</f>
@@ -4435,7 +4505,7 @@
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="34" t="inlineStr">
         <is>
-          <t>TI-D05</t>
+          <t>TI-D04</t>
         </is>
       </c>
       <c r="B22" s="34" t="inlineStr">
@@ -4450,12 +4520,12 @@
       </c>
       <c r="D22" s="35" t="inlineStr">
         <is>
-          <t>Pacote Office 365</t>
+          <t>Antivírus</t>
         </is>
       </c>
       <c r="E22" s="35" t="inlineStr">
         <is>
-          <t>Licenças de software (conferir nº de licenças x usuários) — RATEIO A DEFINIR</t>
+          <t>Proteção para equipamentos — RATEIO A DEFINIR</t>
         </is>
       </c>
       <c r="F22" s="34" t="inlineStr"/>
@@ -4465,28 +4535,28 @@
         </is>
       </c>
       <c r="H22" s="36" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="I22" s="36" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="J22" s="36" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="K22" s="36" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="L22" s="36" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="M22" s="36" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="N22" s="36" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="O22" s="36" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="P22" s="41">
         <f>SUM(H22:O22)</f>
@@ -4496,7 +4566,7 @@
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="34" t="inlineStr">
         <is>
-          <t>TI-D06</t>
+          <t>TI-D05</t>
         </is>
       </c>
       <c r="B23" s="34" t="inlineStr">
@@ -4511,43 +4581,43 @@
       </c>
       <c r="D23" s="35" t="inlineStr">
         <is>
-          <t>Projeto Melhoria de Infraestrutura - Sala de Reunião</t>
+          <t>Pacote Office 365</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Cadeiras, cafeteira, copos, canetas, blocos personalizados, câmeras, microfones etc.</t>
+          <t>Licenças de software (conferir nº de licenças x usuários) — RATEIO A DEFINIR</t>
         </is>
       </c>
       <c r="F23" s="34" t="inlineStr"/>
       <c r="G23" s="34" t="inlineStr">
         <is>
-          <t>Móveis e Utensílios</t>
+          <t>Licenças de Softwares</t>
         </is>
       </c>
       <c r="H23" s="36" t="n">
-        <v>2800</v>
+        <v>375</v>
       </c>
       <c r="I23" s="36" t="n">
-        <v>2800</v>
+        <v>375</v>
       </c>
       <c r="J23" s="36" t="n">
-        <v>2800</v>
+        <v>375</v>
       </c>
       <c r="K23" s="36" t="n">
-        <v>2800</v>
+        <v>375</v>
       </c>
       <c r="L23" s="36" t="n">
-        <v>2800</v>
+        <v>375</v>
       </c>
       <c r="M23" s="36" t="n">
-        <v>2800</v>
+        <v>375</v>
       </c>
       <c r="N23" s="36" t="n">
-        <v>2800</v>
+        <v>375</v>
       </c>
       <c r="O23" s="36" t="n">
-        <v>2800</v>
+        <v>375</v>
       </c>
       <c r="P23" s="41">
         <f>SUM(H23:O23)</f>
@@ -4557,7 +4627,7 @@
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="34" t="inlineStr">
         <is>
-          <t>TI-D07</t>
+          <t>TI-D06</t>
         </is>
       </c>
       <c r="B24" s="34" t="inlineStr">
@@ -4572,39 +4642,43 @@
       </c>
       <c r="D24" s="35" t="inlineStr">
         <is>
-          <t>Cursos e Treinamentos</t>
-        </is>
-      </c>
-      <c r="E24" s="35" t="inlineStr"/>
+          <t>Projeto Melhoria de Infraestrutura - Sala de Reunião</t>
+        </is>
+      </c>
+      <c r="E24" s="35" t="inlineStr">
+        <is>
+          <t>Cadeiras, cafeteira, copos, canetas, blocos personalizados, câmeras, microfones etc.</t>
+        </is>
+      </c>
       <c r="F24" s="34" t="inlineStr"/>
       <c r="G24" s="34" t="inlineStr">
         <is>
-          <t>Custeio de Treinamento</t>
+          <t>Móveis e Utensílios</t>
         </is>
       </c>
       <c r="H24" s="36" t="n">
-        <v>200</v>
+        <v>2800</v>
       </c>
       <c r="I24" s="36" t="n">
-        <v>200</v>
+        <v>2800</v>
       </c>
       <c r="J24" s="36" t="n">
-        <v>200</v>
+        <v>2800</v>
       </c>
       <c r="K24" s="36" t="n">
-        <v>200</v>
+        <v>2800</v>
       </c>
       <c r="L24" s="36" t="n">
-        <v>200</v>
+        <v>2800</v>
       </c>
       <c r="M24" s="36" t="n">
-        <v>200</v>
+        <v>2800</v>
       </c>
       <c r="N24" s="36" t="n">
-        <v>200</v>
+        <v>2800</v>
       </c>
       <c r="O24" s="36" t="n">
-        <v>200</v>
+        <v>2800</v>
       </c>
       <c r="P24" s="41">
         <f>SUM(H24:O24)</f>
@@ -4614,7 +4688,7 @@
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="34" t="inlineStr">
         <is>
-          <t>TI-D08</t>
+          <t>TI-D07</t>
         </is>
       </c>
       <c r="B25" s="34" t="inlineStr">
@@ -4629,39 +4703,39 @@
       </c>
       <c r="D25" s="35" t="inlineStr">
         <is>
-          <t>Aplicativo de Gravação de Reunião</t>
+          <t>Cursos e Treinamentos</t>
         </is>
       </c>
       <c r="E25" s="35" t="inlineStr"/>
       <c r="F25" s="34" t="inlineStr"/>
       <c r="G25" s="34" t="inlineStr">
         <is>
-          <t>Licenças de Softwares</t>
+          <t>Custeio de Treinamento</t>
         </is>
       </c>
       <c r="H25" s="36" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="I25" s="36" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="J25" s="36" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="K25" s="36" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="L25" s="36" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="M25" s="36" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="N25" s="36" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="O25" s="36" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="P25" s="41">
         <f>SUM(H25:O25)</f>
@@ -4671,7 +4745,7 @@
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="34" t="inlineStr">
         <is>
-          <t>TI-D09</t>
+          <t>TI-D08</t>
         </is>
       </c>
       <c r="B26" s="34" t="inlineStr">
@@ -4686,100 +4760,157 @@
       </c>
       <c r="D26" s="35" t="inlineStr">
         <is>
-          <t>Bonificação do time</t>
-        </is>
-      </c>
-      <c r="E26" s="35" t="inlineStr">
-        <is>
-          <t>Cumprimento de prazos e participação em projetos</t>
-        </is>
-      </c>
+          <t>Aplicativo de Gravação de Reunião</t>
+        </is>
+      </c>
+      <c r="E26" s="35" t="inlineStr"/>
       <c r="F26" s="34" t="inlineStr"/>
       <c r="G26" s="34" t="inlineStr">
         <is>
-          <t>Prêmios</t>
+          <t>Licenças de Softwares</t>
         </is>
       </c>
       <c r="H26" s="36" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="I26" s="36" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="J26" s="36" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="K26" s="36" t="n">
-        <v>2400</v>
+        <v>220</v>
       </c>
       <c r="L26" s="36" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="M26" s="36" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="N26" s="36" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="O26" s="36" t="n">
-        <v>3600</v>
+        <v>220</v>
       </c>
       <c r="P26" s="41">
         <f>SUM(H26:O26)</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="34" t="inlineStr">
+        <is>
+          <t>TI-D09</t>
+        </is>
+      </c>
+      <c r="B27" s="34" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="C27" s="34" t="inlineStr">
+        <is>
+          <t>Despesas</t>
+        </is>
+      </c>
+      <c r="D27" s="35" t="inlineStr">
+        <is>
+          <t>Bonificação do time</t>
+        </is>
+      </c>
+      <c r="E27" s="35" t="inlineStr">
+        <is>
+          <t>Cumprimento de prazos e participação em projetos</t>
+        </is>
+      </c>
+      <c r="F27" s="34" t="inlineStr"/>
+      <c r="G27" s="34" t="inlineStr">
+        <is>
+          <t>Prêmios</t>
+        </is>
+      </c>
+      <c r="H27" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="36" t="n">
+        <v>2400</v>
+      </c>
+      <c r="L27" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="36" t="n">
+        <v>3600</v>
+      </c>
+      <c r="P27" s="41">
+        <f>SUM(H27:O27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="15" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="15" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="15" t="n"/>
-      <c r="H27" s="16">
-        <f>SUM(H5:H26)</f>
-        <v/>
-      </c>
-      <c r="I27" s="16">
-        <f>SUM(I5:I26)</f>
-        <v/>
-      </c>
-      <c r="J27" s="16">
-        <f>SUM(J5:J26)</f>
-        <v/>
-      </c>
-      <c r="K27" s="16">
-        <f>SUM(K5:K26)</f>
-        <v/>
-      </c>
-      <c r="L27" s="16">
-        <f>SUM(L5:L26)</f>
-        <v/>
-      </c>
-      <c r="M27" s="16">
-        <f>SUM(M5:M26)</f>
-        <v/>
-      </c>
-      <c r="N27" s="16">
-        <f>SUM(N5:N26)</f>
-        <v/>
-      </c>
-      <c r="O27" s="16">
-        <f>SUM(O5:O26)</f>
-        <v/>
-      </c>
-      <c r="P27" s="16">
-        <f>SUM(P5:P26)</f>
+      <c r="B28" s="15" t="n"/>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="15" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="16">
+        <f>SUM(H5:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="16">
+        <f>SUM(I5:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="16">
+        <f>SUM(J5:J27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="16">
+        <f>SUM(K5:K27)</f>
+        <v/>
+      </c>
+      <c r="L28" s="16">
+        <f>SUM(L5:L27)</f>
+        <v/>
+      </c>
+      <c r="M28" s="16">
+        <f>SUM(M5:M27)</f>
+        <v/>
+      </c>
+      <c r="N28" s="16">
+        <f>SUM(N5:N27)</f>
+        <v/>
+      </c>
+      <c r="O28" s="16">
+        <f>SUM(O5:O27)</f>
+        <v/>
+      </c>
+      <c r="P28" s="16">
+        <f>SUM(P5:P27)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P26"/>
+  <autoFilter ref="A4:P27"/>
   <mergeCells count="2">
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
@@ -4794,7 +4925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5508,9 +5639,15 @@
         <f>Planejado!G15</f>
         <v/>
       </c>
-      <c r="H15" s="45" t="n"/>
-      <c r="I15" s="45" t="n"/>
-      <c r="J15" s="45" t="n"/>
+      <c r="H15" s="45" t="n">
+        <v>2570.52</v>
+      </c>
+      <c r="I15" s="45" t="n">
+        <v>2570.52</v>
+      </c>
+      <c r="J15" s="45" t="n">
+        <v>2570.52</v>
+      </c>
       <c r="K15" s="45" t="n"/>
       <c r="L15" s="45" t="n"/>
       <c r="M15" s="45" t="n"/>
@@ -5520,8 +5657,16 @@
         <f>SUM(H15:O15)</f>
         <v/>
       </c>
-      <c r="Q15" s="46" t="n"/>
-      <c r="R15" s="46" t="n"/>
+      <c r="Q15" s="46" t="inlineStr">
+        <is>
+          <t>Gestora, 05/08/26</t>
+        </is>
+      </c>
+      <c r="R15" s="46" t="inlineStr">
+        <is>
+          <t>Salário bruto vigente até jul; sobe para R$ 3.070,52 em ago</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="43">
@@ -5565,7 +5710,11 @@
         <v/>
       </c>
       <c r="Q16" s="46" t="n"/>
-      <c r="R16" s="46" t="n"/>
+      <c r="R16" s="46" t="inlineStr">
+        <is>
+          <t>PREENCHER — encargos e benefícios sobre o bruto</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="43">
@@ -5596,9 +5745,15 @@
         <f>Planejado!G17</f>
         <v/>
       </c>
-      <c r="H17" s="45" t="n"/>
-      <c r="I17" s="45" t="n"/>
-      <c r="J17" s="45" t="n"/>
+      <c r="H17" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="45" t="n">
+        <v>0</v>
+      </c>
       <c r="K17" s="45" t="n"/>
       <c r="L17" s="45" t="n"/>
       <c r="M17" s="45" t="n"/>
@@ -5608,8 +5763,16 @@
         <f>SUM(H17:O17)</f>
         <v/>
       </c>
-      <c r="Q17" s="46" t="n"/>
-      <c r="R17" s="46" t="n"/>
+      <c r="Q17" s="46" t="inlineStr">
+        <is>
+          <t>Gestora, 05/08/26</t>
+        </is>
+      </c>
+      <c r="R17" s="46" t="inlineStr">
+        <is>
+          <t>Sem acionamento no período — confirmar se o contrato segue ativo</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="43">
@@ -5640,9 +5803,15 @@
         <f>Planejado!G18</f>
         <v/>
       </c>
-      <c r="H18" s="45" t="n"/>
-      <c r="I18" s="45" t="n"/>
-      <c r="J18" s="45" t="n"/>
+      <c r="H18" s="45" t="n">
+        <v>6300</v>
+      </c>
+      <c r="I18" s="45" t="n">
+        <v>6300</v>
+      </c>
+      <c r="J18" s="45" t="n">
+        <v>6300</v>
+      </c>
       <c r="K18" s="45" t="n"/>
       <c r="L18" s="45" t="n"/>
       <c r="M18" s="45" t="n"/>
@@ -5652,8 +5821,16 @@
         <f>SUM(H18:O18)</f>
         <v/>
       </c>
-      <c r="Q18" s="46" t="n"/>
-      <c r="R18" s="46" t="n"/>
+      <c r="Q18" s="46" t="inlineStr">
+        <is>
+          <t>Gestora, 05/08/26</t>
+        </is>
+      </c>
+      <c r="R18" s="46" t="inlineStr">
+        <is>
+          <t>R$ 3.700/mês abaixo do contratado — confirmar escopo</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="43">
@@ -6007,56 +6184,100 @@
       <c r="Q26" s="46" t="n"/>
       <c r="R26" s="46" t="n"/>
     </row>
-    <row r="27">
-      <c r="A27" s="47" t="inlineStr">
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="43">
+        <f>Planejado!A27</f>
+        <v/>
+      </c>
+      <c r="B27" s="43">
+        <f>Planejado!B27</f>
+        <v/>
+      </c>
+      <c r="C27" s="43">
+        <f>Planejado!C27</f>
+        <v/>
+      </c>
+      <c r="D27" s="44">
+        <f>Planejado!D27</f>
+        <v/>
+      </c>
+      <c r="E27" s="44">
+        <f>Planejado!E27</f>
+        <v/>
+      </c>
+      <c r="F27" s="43">
+        <f>Planejado!F27</f>
+        <v/>
+      </c>
+      <c r="G27" s="43">
+        <f>Planejado!G27</f>
+        <v/>
+      </c>
+      <c r="H27" s="45" t="n"/>
+      <c r="I27" s="45" t="n"/>
+      <c r="J27" s="45" t="n"/>
+      <c r="K27" s="45" t="n"/>
+      <c r="L27" s="45" t="n"/>
+      <c r="M27" s="45" t="n"/>
+      <c r="N27" s="45" t="n"/>
+      <c r="O27" s="45" t="n"/>
+      <c r="P27" s="41">
+        <f>SUM(H27:O27)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="46" t="n"/>
+      <c r="R27" s="46" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="47" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B27" s="47" t="n"/>
-      <c r="C27" s="47" t="n"/>
-      <c r="D27" s="47" t="n"/>
-      <c r="E27" s="47" t="n"/>
-      <c r="F27" s="47" t="n"/>
-      <c r="G27" s="47" t="n"/>
-      <c r="H27" s="48">
-        <f>SUM(H5:H26)</f>
-        <v/>
-      </c>
-      <c r="I27" s="48">
-        <f>SUM(I5:I26)</f>
-        <v/>
-      </c>
-      <c r="J27" s="48">
-        <f>SUM(J5:J26)</f>
-        <v/>
-      </c>
-      <c r="K27" s="48">
-        <f>SUM(K5:K26)</f>
-        <v/>
-      </c>
-      <c r="L27" s="48">
-        <f>SUM(L5:L26)</f>
-        <v/>
-      </c>
-      <c r="M27" s="48">
-        <f>SUM(M5:M26)</f>
-        <v/>
-      </c>
-      <c r="N27" s="48">
-        <f>SUM(N5:N26)</f>
-        <v/>
-      </c>
-      <c r="O27" s="48">
-        <f>SUM(O5:O26)</f>
-        <v/>
-      </c>
-      <c r="P27" s="48">
-        <f>SUM(P5:P26)</f>
-        <v/>
-      </c>
-      <c r="Q27" s="47" t="n"/>
-      <c r="R27" s="47" t="n"/>
+      <c r="B28" s="47" t="n"/>
+      <c r="C28" s="47" t="n"/>
+      <c r="D28" s="47" t="n"/>
+      <c r="E28" s="47" t="n"/>
+      <c r="F28" s="47" t="n"/>
+      <c r="G28" s="47" t="n"/>
+      <c r="H28" s="48">
+        <f>SUM(H5:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="48">
+        <f>SUM(I5:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="48">
+        <f>SUM(J5:J27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="48">
+        <f>SUM(K5:K27)</f>
+        <v/>
+      </c>
+      <c r="L28" s="48">
+        <f>SUM(L5:L27)</f>
+        <v/>
+      </c>
+      <c r="M28" s="48">
+        <f>SUM(M5:M27)</f>
+        <v/>
+      </c>
+      <c r="N28" s="48">
+        <f>SUM(N5:N27)</f>
+        <v/>
+      </c>
+      <c r="O28" s="48">
+        <f>SUM(O5:O27)</f>
+        <v/>
+      </c>
+      <c r="P28" s="48">
+        <f>SUM(P5:P27)</f>
+        <v/>
+      </c>
+      <c r="Q28" s="47" t="n"/>
+      <c r="R28" s="47" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6161,19 +6382,19 @@
         </is>
       </c>
       <c r="B5" s="30">
-        <f>SUMIFS(Planejado!$H$5:$H$26,Planejado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$H$5:$H$27,Planejado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="C5" s="30">
-        <f>SUMIFS(Realizado!$H$5:$H$26,Realizado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$H$5:$H$27,Realizado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="D5" s="30">
-        <f>SUMIFS(Planejado!$H$5:$H$26,Planejado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Planejado!$H$5:$H$27,Planejado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="E5" s="30">
-        <f>SUMIFS(Realizado!$H$5:$H$26,Realizado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Realizado!$H$5:$H$27,Realizado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="F5" s="30">
@@ -6204,19 +6425,19 @@
         </is>
       </c>
       <c r="B6" s="36">
-        <f>SUMIFS(Planejado!$I$5:$I$26,Planejado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$I$5:$I$27,Planejado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="C6" s="36">
-        <f>SUMIFS(Realizado!$I$5:$I$26,Realizado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$I$5:$I$27,Realizado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="D6" s="36">
-        <f>SUMIFS(Planejado!$I$5:$I$26,Planejado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Planejado!$I$5:$I$27,Planejado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="E6" s="36">
-        <f>SUMIFS(Realizado!$I$5:$I$26,Realizado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Realizado!$I$5:$I$27,Realizado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="F6" s="36">
@@ -6247,19 +6468,19 @@
         </is>
       </c>
       <c r="B7" s="30">
-        <f>SUMIFS(Planejado!$J$5:$J$26,Planejado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$J$5:$J$27,Planejado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="C7" s="30">
-        <f>SUMIFS(Realizado!$J$5:$J$26,Realizado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$J$5:$J$27,Realizado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="D7" s="30">
-        <f>SUMIFS(Planejado!$J$5:$J$26,Planejado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Planejado!$J$5:$J$27,Planejado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="E7" s="30">
-        <f>SUMIFS(Realizado!$J$5:$J$26,Realizado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Realizado!$J$5:$J$27,Realizado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="F7" s="30">
@@ -6290,19 +6511,19 @@
         </is>
       </c>
       <c r="B8" s="36">
-        <f>SUMIFS(Planejado!$K$5:$K$26,Planejado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$K$5:$K$27,Planejado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="C8" s="36">
-        <f>SUMIFS(Realizado!$K$5:$K$26,Realizado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$K$5:$K$27,Realizado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="D8" s="36">
-        <f>SUMIFS(Planejado!$K$5:$K$26,Planejado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Planejado!$K$5:$K$27,Planejado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="E8" s="36">
-        <f>SUMIFS(Realizado!$K$5:$K$26,Realizado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Realizado!$K$5:$K$27,Realizado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="F8" s="36">
@@ -6333,19 +6554,19 @@
         </is>
       </c>
       <c r="B9" s="30">
-        <f>SUMIFS(Planejado!$L$5:$L$26,Planejado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$L$5:$L$27,Planejado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="C9" s="30">
-        <f>SUMIFS(Realizado!$L$5:$L$26,Realizado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$L$5:$L$27,Realizado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="D9" s="30">
-        <f>SUMIFS(Planejado!$L$5:$L$26,Planejado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Planejado!$L$5:$L$27,Planejado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="E9" s="30">
-        <f>SUMIFS(Realizado!$L$5:$L$26,Realizado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Realizado!$L$5:$L$27,Realizado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="F9" s="30">
@@ -6376,19 +6597,19 @@
         </is>
       </c>
       <c r="B10" s="36">
-        <f>SUMIFS(Planejado!$M$5:$M$26,Planejado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$M$5:$M$27,Planejado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="C10" s="36">
-        <f>SUMIFS(Realizado!$M$5:$M$26,Realizado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$M$5:$M$27,Realizado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="D10" s="36">
-        <f>SUMIFS(Planejado!$M$5:$M$26,Planejado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Planejado!$M$5:$M$27,Planejado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="E10" s="36">
-        <f>SUMIFS(Realizado!$M$5:$M$26,Realizado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Realizado!$M$5:$M$27,Realizado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="F10" s="36">
@@ -6419,19 +6640,19 @@
         </is>
       </c>
       <c r="B11" s="30">
-        <f>SUMIFS(Planejado!$N$5:$N$26,Planejado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$N$5:$N$27,Planejado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="C11" s="30">
-        <f>SUMIFS(Realizado!$N$5:$N$26,Realizado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$N$5:$N$27,Realizado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="D11" s="30">
-        <f>SUMIFS(Planejado!$N$5:$N$26,Planejado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Planejado!$N$5:$N$27,Planejado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="E11" s="30">
-        <f>SUMIFS(Realizado!$N$5:$N$26,Realizado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Realizado!$N$5:$N$27,Realizado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="F11" s="30">
@@ -6462,19 +6683,19 @@
         </is>
       </c>
       <c r="B12" s="36">
-        <f>SUMIFS(Planejado!$O$5:$O$26,Planejado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$O$5:$O$27,Planejado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="C12" s="36">
-        <f>SUMIFS(Realizado!$O$5:$O$26,Realizado!$B$5:$B$26,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$O$5:$O$27,Realizado!$B$5:$B$27,"Jurídico")</f>
         <v/>
       </c>
       <c r="D12" s="36">
-        <f>SUMIFS(Planejado!$O$5:$O$26,Planejado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Planejado!$O$5:$O$27,Planejado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="E12" s="36">
-        <f>SUMIFS(Realizado!$O$5:$O$26,Realizado!$B$5:$B$26,"TI")</f>
+        <f>SUMIFS(Realizado!$O$5:$O$27,Realizado!$B$5:$B$27,"TI")</f>
         <v/>
       </c>
       <c r="F12" s="36">
@@ -6647,19 +6868,19 @@
         </is>
       </c>
       <c r="B5" s="30">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A5,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A5,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="C5" s="30">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A5,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A5,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="D5" s="30">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A5,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A5,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="E5" s="30">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A5,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A5,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="F5" s="30">
@@ -6679,7 +6900,7 @@
         <v/>
       </c>
       <c r="J5" s="30">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$G$5:$G$26,$A5)</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$G$5:$G$27,$A5)</f>
         <v/>
       </c>
     </row>
@@ -6690,19 +6911,19 @@
         </is>
       </c>
       <c r="B6" s="36">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A6,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A6,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="C6" s="36">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A6,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A6,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="D6" s="36">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A6,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A6,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="E6" s="36">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A6,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A6,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="F6" s="36">
@@ -6722,7 +6943,7 @@
         <v/>
       </c>
       <c r="J6" s="36">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$G$5:$G$26,$A6)</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$G$5:$G$27,$A6)</f>
         <v/>
       </c>
     </row>
@@ -6733,19 +6954,19 @@
         </is>
       </c>
       <c r="B7" s="30">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A7,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A7,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="C7" s="30">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A7,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A7,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="D7" s="30">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A7,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A7,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="E7" s="30">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A7,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A7,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="F7" s="30">
@@ -6765,7 +6986,7 @@
         <v/>
       </c>
       <c r="J7" s="30">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$G$5:$G$26,$A7)</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$G$5:$G$27,$A7)</f>
         <v/>
       </c>
     </row>
@@ -6776,19 +6997,19 @@
         </is>
       </c>
       <c r="B8" s="36">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A8,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A8,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="C8" s="36">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A8,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A8,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="D8" s="36">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A8,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A8,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="E8" s="36">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A8,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A8,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="F8" s="36">
@@ -6808,7 +7029,7 @@
         <v/>
       </c>
       <c r="J8" s="36">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$G$5:$G$26,$A8)</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$G$5:$G$27,$A8)</f>
         <v/>
       </c>
     </row>
@@ -6819,19 +7040,19 @@
         </is>
       </c>
       <c r="B9" s="30">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A9,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A9,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="C9" s="30">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A9,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A9,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="D9" s="30">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A9,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A9,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="E9" s="30">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A9,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A9,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="F9" s="30">
@@ -6851,7 +7072,7 @@
         <v/>
       </c>
       <c r="J9" s="30">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$G$5:$G$26,$A9)</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$G$5:$G$27,$A9)</f>
         <v/>
       </c>
     </row>
@@ -6862,19 +7083,19 @@
         </is>
       </c>
       <c r="B10" s="36">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A10,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A10,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="C10" s="36">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A10,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A10,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="D10" s="36">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A10,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A10,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="E10" s="36">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A10,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A10,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="F10" s="36">
@@ -6894,7 +7115,7 @@
         <v/>
       </c>
       <c r="J10" s="36">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$G$5:$G$26,$A10)</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$G$5:$G$27,$A10)</f>
         <v/>
       </c>
     </row>
@@ -6905,19 +7126,19 @@
         </is>
       </c>
       <c r="B11" s="30">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A11,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A11,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="C11" s="30">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A11,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A11,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="D11" s="30">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A11,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A11,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="E11" s="30">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A11,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A11,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="F11" s="30">
@@ -6937,7 +7158,7 @@
         <v/>
       </c>
       <c r="J11" s="30">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$G$5:$G$26,$A11)</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$G$5:$G$27,$A11)</f>
         <v/>
       </c>
     </row>
@@ -6948,19 +7169,19 @@
         </is>
       </c>
       <c r="B12" s="36">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A12,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A12,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="C12" s="36">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A12,Comparativo!$B$6:$B$27,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A12,Comparativo!$B$6:$B$28,"Jurídico")</f>
         <v/>
       </c>
       <c r="D12" s="36">
-        <f>SUMIFS(Comparativo!$I$6:$I$27,Comparativo!$E$6:$E$27,$A12,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$28,Comparativo!$E$6:$E$28,$A12,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="E12" s="36">
-        <f>SUMIFS(Comparativo!$J$6:$J$27,Comparativo!$E$6:$E$27,$A12,Comparativo!$B$6:$B$27,"TI")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$28,Comparativo!$E$6:$E$28,$A12,Comparativo!$B$6:$B$28,"TI")</f>
         <v/>
       </c>
       <c r="F12" s="36">
@@ -6980,7 +7201,7 @@
         <v/>
       </c>
       <c r="J12" s="36">
-        <f>SUMIFS(Planejado!$P$5:$P$26,Planejado!$G$5:$G$26,$A12)</f>
+        <f>SUMIFS(Planejado!$P$5:$P$27,Planejado!$G$5:$G$27,$A12)</f>
         <v/>
       </c>
     </row>
@@ -7050,7 +7271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7147,17 +7368,17 @@
       </c>
       <c r="B6" s="59" t="inlineStr">
         <is>
-          <t>Vinicius Di Franco tem o mesmo problema</t>
+          <t>Encargos do Vinicius — CAMPO A PREENCHER</t>
         </is>
       </c>
       <c r="C6" s="59" t="inlineStr">
         <is>
-          <t>O orçamento dele (R$ 5.416,53/mês) também é custo total com encargos. Quando o realizado do TI for lançado, ou vem o custo total, ou a linha precisa ser dividida em bruto + encargos como foi feito com a Geovanna.</t>
+          <t>A linha TI-E01B foi criada para receber os encargos e benefícios sobre o salário bruto, mesmo tratamento dado à Geovanna. Hoje está em branco. Aumento permanente de R$ 500 registrado a partir de 05/08/26 (bruto de R$ 2.570,52 para R$ 3.070,52), o que eleva o orçamento em R$ 2.500 no restante do ano.</t>
         </is>
       </c>
       <c r="D6" s="59" t="inlineStr">
         <is>
-          <t>Se lançarem o bruto contra o orçado de custo total, o TI vai mostrar uma economia falsa da mesma natureza.</t>
+          <t>Enquanto não for preenchida, a folha do TI aparece R$ 2.846,01/mês abaixo do orçado — economia que não existe. Atenção: o orçado de custo total (R$ 5.416,53) implica encargos de 111% sobre o bruto de R$ 2.570,52, bem acima do usual (67% a 80%) — vale conferir se o orçamento dele está folgado.</t>
         </is>
       </c>
       <c r="E6" s="59" t="inlineStr">
@@ -7165,31 +7386,31 @@
           <t>Cristiane + RH</t>
         </is>
       </c>
-      <c r="F6" s="60" t="inlineStr">
-        <is>
-          <t>EM ABERTO</t>
+      <c r="F6" s="57" t="inlineStr">
+        <is>
+          <t>PREENCHER</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="55" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B7" s="56" t="inlineStr">
         <is>
-          <t>Reajuste da Thamar — revisão orçamentária</t>
+          <t>Jonathan R$ 3.700/mês abaixo do contratado</t>
         </is>
       </c>
       <c r="C7" s="56" t="inlineStr">
         <is>
-          <t>Reajuste permanente de R$ 5.000 para R$ 5.500/mês, já em vigor desde mai/26. O planejado foi mantido em R$ 5.000 em mai–set (para o desvio ficar visível) e revisado para R$ 5.500 de out a dez.</t>
+          <t>Orçado R$ 10.000/mês, realizado R$ 6.300/mês em mai, jun e jul.</t>
         </is>
       </c>
       <c r="D7" s="56" t="inlineStr">
         <is>
-          <t>Desvio já incorrido de R$ 500/mês. Impacto de +R$ 1.500 no orçamento do restante do ano; o orçamento total sobe para R$ 395.852,68.</t>
+          <t>Maior desvio em reais de todo o orçamento: R$ 11.100 em três meses. Se o valor menor for o novo padrão, o planejado de ago a dez deve ser revisado para baixo — sobrariam R$ 18.500 no orçamento do TI.</t>
         </is>
       </c>
       <c r="E7" s="56" t="inlineStr">
@@ -7197,31 +7418,31 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F7" s="61" t="inlineStr">
-        <is>
-          <t>APLICADO</t>
+      <c r="F7" s="60" t="inlineStr">
+        <is>
+          <t>EM ABERTO</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="58" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="B8" s="59" t="inlineStr">
         <is>
-          <t>Jusbrasil 30% acima do orçado</t>
+          <t>Elias Benedito zerado nos três meses</t>
         </is>
       </c>
       <c r="C8" s="59" t="inlineStr">
         <is>
-          <t>Orçado R$ 104,90/mês, realizado R$ 136,00/mês nos três meses.</t>
+          <t>Orçado R$ 1.065/mês como suporte técnico terceirizado, realizado R$ 0 em mai, jun e jul.</t>
         </is>
       </c>
       <c r="D8" s="59" t="inlineStr">
         <is>
-          <t>Menor desvio em reais (R$ 31,10/mês), mas o maior em percentual. Vale conferir se houve reajuste contratual ou mudança de plano.</t>
+          <t>Confirmar se o contrato segue ativo (acionamento sob demanda) ou se foi encerrado. Se encerrado, são R$ 8.520 a liberar no orçamento do ano.</t>
         </is>
       </c>
       <c r="E8" s="59" t="inlineStr">
@@ -7238,22 +7459,22 @@
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="55" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B9" s="56" t="inlineStr">
         <is>
-          <t>Bonificação de ago/26 do Jurídico</t>
+          <t>Reajuste da Thamar — revisão orçamentária</t>
         </is>
       </c>
       <c r="C9" s="56" t="inlineStr">
         <is>
-          <t>Estão orçados R$ 10.293,60 em agosto e R$ 12.867,00 em dezembro. O realizado de agosto ainda não foi informado.</t>
+          <t>Reajuste permanente de R$ 5.000 para R$ 5.500/mês, já em vigor desde mai/26. O planejado foi mantido em R$ 5.000 em mai–set (para o desvio ficar visível) e revisado para R$ 5.500 de out a dez.</t>
         </is>
       </c>
       <c r="D9" s="56" t="inlineStr">
         <is>
-          <t>É a maior despesa isolada do Jurídico no segundo semestre. Sem confirmação, o acumulado de agosto fica distorcido.</t>
+          <t>Desvio já incorrido de R$ 500/mês. Impacto de +R$ 1.500 no orçamento do restante do ano; o orçamento total sobe para R$ 395.852,68.</t>
         </is>
       </c>
       <c r="E9" s="56" t="inlineStr">
@@ -7261,31 +7482,31 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F9" s="60" t="inlineStr">
-        <is>
-          <t>EM ABERTO</t>
+      <c r="F9" s="61" t="inlineStr">
+        <is>
+          <t>APLICADO</t>
         </is>
       </c>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B10" s="59" t="inlineStr">
         <is>
-          <t>Base de meses do time de TI</t>
+          <t>Jusbrasil 30% acima do orçado</t>
         </is>
       </c>
       <c r="C10" s="59" t="inlineStr">
         <is>
-          <t>A ficha original trazia a coluna TOTAL do TI em bases diferentes por pessoa (Vinicius e Elias em 12 meses, Jonathan em 9), enquanto o grid mensal tem 8 (mai–dez). Definido: vale mai–dez para todos.</t>
+          <t>Orçado R$ 104,90/mês, realizado R$ 136,00/mês nos três meses.</t>
         </is>
       </c>
       <c r="D10" s="59" t="inlineStr">
         <is>
-          <t>Orçamento de equipe do TI passou de R$ 167.778,30 para R$ 131.852,20 (−R$ 35.926,10). Total geral: R$ 394.352,68.</t>
+          <t>Menor desvio em reais (R$ 31,10/mês), mas o maior em percentual. Vale conferir se houve reajuste contratual ou mudança de plano.</t>
         </is>
       </c>
       <c r="E10" s="59" t="inlineStr">
@@ -7293,36 +7514,36 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F10" s="61" t="inlineStr">
-        <is>
-          <t>RESOLVIDO</t>
+      <c r="F10" s="60" t="inlineStr">
+        <is>
+          <t>EM ABERTO</t>
         </is>
       </c>
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="55" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>E</t>
         </is>
       </c>
       <c r="B11" s="56" t="inlineStr">
         <is>
-          <t>Origem do valor realizado</t>
+          <t>Bonificação de ago/26 do Jurídico</t>
         </is>
       </c>
       <c r="C11" s="56" t="inlineStr">
         <is>
-          <t>Ainda não definido se o realizado virá de lançamento manual, de relatório do financeiro/ERP por centro de custo, ou misto.</t>
+          <t>Estão orçados R$ 10.293,60 em agosto e R$ 12.867,00 em dezembro. O realizado de agosto ainda não foi informado.</t>
         </is>
       </c>
       <c r="D11" s="56" t="inlineStr">
         <is>
-          <t>Sem fonte definida o realizado pode divergir da contabilidade e o comparativo perde valor na apresentação à diretoria.</t>
+          <t>É a maior despesa isolada do Jurídico no segundo semestre. Sem confirmação, o acumulado de agosto fica distorcido.</t>
         </is>
       </c>
       <c r="E11" s="56" t="inlineStr">
         <is>
-          <t>Cristiane + Financeiro</t>
+          <t>Cristiane</t>
         </is>
       </c>
       <c r="F11" s="60" t="inlineStr">
@@ -7334,22 +7555,22 @@
     <row r="12" ht="58" customHeight="1">
       <c r="A12" s="58" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B12" s="59" t="inlineStr">
         <is>
-          <t>Jusfy x Astrea</t>
+          <t>Base de meses do time de TI</t>
         </is>
       </c>
       <c r="C12" s="59" t="inlineStr">
         <is>
-          <t>O risco era pagar os dois em paralelo. O realizado de mai–jul mostra Astrea em R$ 0 (cancelado) e Jusfy em R$ 0 (ainda não iniciado) — no momento não há custo de nenhum dos dois.</t>
+          <t>A ficha original trazia a coluna TOTAL do TI em bases diferentes por pessoa (Vinicius e Elias em 12 meses, Jonathan em 9), enquanto o grid mensal tem 8 (mai–dez). Definido: vale mai–dez para todos.</t>
         </is>
       </c>
       <c r="D12" s="59" t="inlineStr">
         <is>
-          <t>Economia de R$ 212,07/mês enquanto durar. Falta decidir se o Jusfy entra e quando, para ajustar o planejado de ago a dez.</t>
+          <t>Orçamento de equipe do TI passou de R$ 167.778,30 para R$ 131.852,20 (−R$ 35.926,10). Total geral: R$ 394.352,68.</t>
         </is>
       </c>
       <c r="E12" s="59" t="inlineStr">
@@ -7366,27 +7587,27 @@
     <row r="13" ht="58" customHeight="1">
       <c r="A13" s="55" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B13" s="56" t="inlineStr">
         <is>
-          <t>Rateio dos softwares corporativos de TI</t>
+          <t>Origem do valor realizado</t>
         </is>
       </c>
       <c r="C13" s="56" t="inlineStr">
         <is>
-          <t>Backup (R$ 6.600), Adapta/IA (R$ 12.200), Antivírus (R$ 1.920) e Office 365 (R$ 3.000) estão marcados na ficha como 'não sei se seria administrativo'. Total: R$ 23.720.</t>
+          <t>Ainda não definido se o realizado virá de lançamento manual, de relatório do financeiro/ERP por centro de custo, ou misto.</t>
         </is>
       </c>
       <c r="D13" s="56" t="inlineStr">
         <is>
-          <t>Se são da empresa toda e ficam no centro de custo de TI, o TI carrega despesa que não é dele e aparece caro no comparativo.</t>
+          <t>Sem fonte definida o realizado pode divergir da contabilidade e o comparativo perde valor na apresentação à diretoria.</t>
         </is>
       </c>
       <c r="E13" s="56" t="inlineStr">
         <is>
-          <t>Cristiane + Controladoria</t>
+          <t>Cristiane + Financeiro</t>
         </is>
       </c>
       <c r="F13" s="60" t="inlineStr">
@@ -7398,22 +7619,22 @@
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="58" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B14" s="59" t="inlineStr">
         <is>
-          <t>Sala de Reunião — recorrente ou pontual?</t>
+          <t>Jusfy x Astrea</t>
         </is>
       </c>
       <c r="C14" s="59" t="inlineStr">
         <is>
-          <t>R$ 2.800/mês × 8 = R$ 22.400 diluídos linearmente, classificados em Móveis e Utensílios.</t>
+          <t>O risco era pagar os dois em paralelo. O realizado de mai–jul mostra Astrea em R$ 0 (cancelado) e Jusfy em R$ 0 (ainda não iniciado) — no momento não há custo de nenhum dos dois.</t>
         </is>
       </c>
       <c r="D14" s="59" t="inlineStr">
         <is>
-          <t>Se for compra pontual (CAPEX), o desvio mensal vai acusar alarme falso todo mês até a compra acontecer, e um pico no mês da compra.</t>
+          <t>Economia de R$ 212,07/mês enquanto durar. Falta decidir se o Jusfy entra e quando, para ajustar o planejado de ago a dez.</t>
         </is>
       </c>
       <c r="E14" s="59" t="inlineStr">
@@ -7421,36 +7642,36 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F14" s="60" t="inlineStr">
-        <is>
-          <t>EM ABERTO</t>
+      <c r="F14" s="61" t="inlineStr">
+        <is>
+          <t>RESOLVIDO</t>
         </is>
       </c>
     </row>
     <row r="15" ht="58" customHeight="1">
       <c r="A15" s="55" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B15" s="56" t="inlineStr">
         <is>
-          <t>Office 365 — nº de licenças</t>
+          <t>Rateio dos softwares corporativos de TI</t>
         </is>
       </c>
       <c r="C15" s="56" t="inlineStr">
         <is>
-          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+          <t>Backup (R$ 6.600), Adapta/IA (R$ 12.200), Antivírus (R$ 1.920) e Office 365 (R$ 3.000) estão marcados na ficha como 'não sei se seria administrativo'. Total: R$ 23.720.</t>
         </is>
       </c>
       <c r="D15" s="56" t="inlineStr">
         <is>
-          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+          <t>Se são da empresa toda e ficam no centro de custo de TI, o TI carrega despesa que não é dele e aparece caro no comparativo.</t>
         </is>
       </c>
       <c r="E15" s="56" t="inlineStr">
         <is>
-          <t>Cristiane</t>
+          <t>Cristiane + Controladoria</t>
         </is>
       </c>
       <c r="F15" s="60" t="inlineStr">
@@ -7462,30 +7683,94 @@
     <row r="16" ht="58" customHeight="1">
       <c r="A16" s="58" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B16" s="59" t="inlineStr">
+        <is>
+          <t>Sala de Reunião — recorrente ou pontual?</t>
+        </is>
+      </c>
+      <c r="C16" s="59" t="inlineStr">
+        <is>
+          <t>R$ 2.800/mês × 8 = R$ 22.400 diluídos linearmente, classificados em Móveis e Utensílios.</t>
+        </is>
+      </c>
+      <c r="D16" s="59" t="inlineStr">
+        <is>
+          <t>Se for compra pontual (CAPEX), o desvio mensal vai acusar alarme falso todo mês até a compra acontecer, e um pico no mês da compra.</t>
+        </is>
+      </c>
+      <c r="E16" s="59" t="inlineStr">
+        <is>
+          <t>Cristiane</t>
+        </is>
+      </c>
+      <c r="F16" s="60" t="inlineStr">
+        <is>
+          <t>EM ABERTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="55" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B17" s="56" t="inlineStr">
+        <is>
+          <t>Office 365 — nº de licenças</t>
+        </is>
+      </c>
+      <c r="C17" s="56" t="inlineStr">
+        <is>
+          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+        </is>
+      </c>
+      <c r="D17" s="56" t="inlineStr">
+        <is>
+          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+        </is>
+      </c>
+      <c r="E17" s="56" t="inlineStr">
+        <is>
+          <t>Cristiane</t>
+        </is>
+      </c>
+      <c r="F17" s="60" t="inlineStr">
+        <is>
+          <t>EM ABERTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="58" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B18" s="59" t="inlineStr">
         <is>
           <t>Critério de competência x caixa</t>
         </is>
       </c>
-      <c r="C16" s="59" t="inlineStr">
+      <c r="C18" s="59" t="inlineStr">
         <is>
           <t>Definir se o realizado será lançado pela data de pagamento (caixa) ou pelo mês de referência da despesa (competência).</t>
         </is>
       </c>
-      <c r="D16" s="59" t="inlineStr">
+      <c r="D18" s="59" t="inlineStr">
         <is>
           <t>Misturar os dois critérios gera desvio artificial em meses de virada, principalmente em folha e prêmios.</t>
         </is>
       </c>
-      <c r="E16" s="59" t="inlineStr">
+      <c r="E18" s="59" t="inlineStr">
         <is>
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F16" s="60" t="inlineStr">
+      <c r="F18" s="60" t="inlineStr">
         <is>
           <t>EM ABERTO</t>
         </is>

</xml_diff>

<commit_message>
docs(orcamento): registra que o orcado do Vinicius tem folga planejada
Gestora confirmou que R$ 2.570,52 (ate jul) e R$ 3.070,52 (de ago) sao
salarios BRUTOS, e que o custo total orcado de R$ 5.416,53 foi
dimensionado prevendo um aumento maior ainda nao concedido.

Isso explica os 111% de encargos implicitos que a aba Pendencias
apontava como suspeitos: nao era erro de orcamento, era folga
proposital. A consequencia pratica muda a leitura do desvio — a folga
nao e economia estrutural e, com o bruto de agosto, praticamente se
esgota.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -4147,7 +4147,7 @@
       </c>
       <c r="E16" s="35" t="inlineStr">
         <is>
-          <t>INSS patronal, FGTS, provisões de 13º e férias, benefícios — PREENCHER</t>
+          <t>INSS patronal, FGTS, provisões de 13º e férias, benefícios — PREENCHER. O orçado de custo total (R$ 5.416,53) foi dimensionado com folga para um aumento futuro ainda não concedido — a folga não é economia estrutural.</t>
         </is>
       </c>
       <c r="F16" s="34" t="inlineStr">
@@ -7373,12 +7373,12 @@
       </c>
       <c r="C6" s="59" t="inlineStr">
         <is>
-          <t>A linha TI-E01B foi criada para receber os encargos e benefícios sobre o salário bruto, mesmo tratamento dado à Geovanna. Hoje está em branco. Aumento permanente de R$ 500 registrado a partir de 05/08/26 (bruto de R$ 2.570,52 para R$ 3.070,52), o que eleva o orçamento em R$ 2.500 no restante do ano.</t>
+          <t>A linha TI-E01B recebe os encargos e benefícios sobre o salário bruto, mesmo tratamento dado à Geovanna. Hoje está em branco. Brutos confirmados pela gestora: R$ 2.570,52 até jul/26 e R$ 3.070,52 a partir de 05/08/26.</t>
         </is>
       </c>
       <c r="D6" s="59" t="inlineStr">
         <is>
-          <t>Enquanto não for preenchida, a folha do TI aparece R$ 2.846,01/mês abaixo do orçado — economia que não existe. Atenção: o orçado de custo total (R$ 5.416,53) implica encargos de 111% sobre o bruto de R$ 2.570,52, bem acima do usual (67% a 80%) — vale conferir se o orçamento dele está folgado.</t>
+          <t>A folga do orçado NÃO é economia estrutural: o custo total de R$ 5.416,53 foi dimensionado prevendo um aumento maior, ainda não concedido. Com o bruto de agosto, a folga praticamente se esgota — a encargos de 67% o custo vai a R$ 5.127,77 (sobram R$ 288,76/mês) e a 80% passa a estourar o orçado. Preencher os encargos reais é o que define se ainda há margem.</t>
         </is>
       </c>
       <c r="E6" s="59" t="inlineStr">

</xml_diff>

<commit_message>
fix(orcamento): aumento do Vinicius e absorvido pela folga, nao somado
O commit anterior elevou o planejado dele em R$ 500/mes de ago a dez,
tratando o aumento como o reajuste da Thamar. Errado: o envelope de
custo total do Vinicius (R$ 5.416,525/mes) ja fora dimensionado
prevendo um aumento, conforme a gestora confirmou. O reajuste consome
a folga existente em vez de criar despesa nova.

O planejado de encargos passa a ser o residuo do envelope (cai
R$ 500 em ago, exatamente o que o bruto subiu), mantendo o custo total
fixo em R$ 5.416,525 nos oito meses.

Equipe de TI volta a R$ 131.852,20 e o total geral a R$ 395.852,68.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -4082,7 +4082,7 @@
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Analista Administrativo — aumento de R$ 2.570,52 para R$ 3.070,52 a partir de 05/08/26</t>
+          <t>Analista Administrativo — aumento de R$ 2.570,52 para R$ 3.070,52 a partir de 05/08/26, absorvido pela folga do envelope orçado (custo total segue R$ 5.416,525/mês)</t>
         </is>
       </c>
       <c r="F15" s="34" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="E16" s="35" t="inlineStr">
         <is>
-          <t>INSS patronal, FGTS, provisões de 13º e férias, benefícios — PREENCHER. O orçado de custo total (R$ 5.416,53) foi dimensionado com folga para um aumento futuro ainda não concedido — a folga não é economia estrutural.</t>
+          <t>INSS patronal, FGTS, provisões de 13º e férias, benefícios — PREENCHER. Planejado = resíduo do envelope de R$ 5.416,525/mês, que já previa o aumento. A folga não é economia estrutural: com o bruto de agosto ela quase se esgota.</t>
         </is>
       </c>
       <c r="F16" s="34" t="inlineStr">
@@ -4170,19 +4170,19 @@
         <v>2846.005</v>
       </c>
       <c r="K16" s="36" t="n">
-        <v>2846.005</v>
+        <v>2346.005</v>
       </c>
       <c r="L16" s="36" t="n">
-        <v>2846.005</v>
+        <v>2346.005</v>
       </c>
       <c r="M16" s="36" t="n">
-        <v>2846.005</v>
+        <v>2346.005</v>
       </c>
       <c r="N16" s="36" t="n">
-        <v>2846.005</v>
+        <v>2346.005</v>
       </c>
       <c r="O16" s="36" t="n">
-        <v>2846.005</v>
+        <v>2346.005</v>
       </c>
       <c r="P16" s="41">
         <f>SUM(H16:O16)</f>

</xml_diff>

<commit_message>
feat(orcamento): planilhas separadas por departamento
Gera uma planilha para o Juridico e outra para o TI, alem do
consolidado. O corpo do gerador virou a funcao gerar(DEPTO, OUT).

Nas planilhas de um departamento so, o Painel, o resumo por plano de
contas e a evolucao mensal se reduzem aquele departamento — as colunas
por area passaram a ser montadas dinamicamente em vez de fixas em
Juridico/TI. A aba Pendencias ganhou um campo de departamento e cada
planilha mostra o que e da sua area mais o que vale para as duas; o
resumo por plano de contas lista so os planos que aquele recorte usa.

Os tres arquivos saem da mesma base e reconciliam:
  Juridico    290.730,42 orcado / 54.932,73 realizado
  TI          256.818,30 orcado / 26.611,56 realizado
  Consolidado 547.548,72 orcado / 81.544,29 realizado

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -161,12 +161,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -1043,7 +1043,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PAINEL EXECUTIVO  —  Orçamento 2026 Jurídico e TI</t>
+          <t>PAINEL EXECUTIVO  —  Orçamento 2026  JURÍDICO E TI</t>
         </is>
       </c>
     </row>
@@ -3364,7 +3364,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ORÇAMENTO PLANEJADO 2026  —  Jurídico e TI</t>
+          <t>ORÇAMENTO PLANEJADO 2026  —  JURÍDICO E TI</t>
         </is>
       </c>
     </row>
@@ -5279,7 +5279,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REALIZADO 2026  —  Jurídico e TI</t>
+          <t>REALIZADO 2026  —  JURÍDICO E TI</t>
         </is>
       </c>
     </row>
@@ -6662,15 +6662,15 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -7320,15 +7320,15 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -7786,8 +7786,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:H12">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -7807,7 +7807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7877,7 +7877,7 @@
       </c>
       <c r="C5" s="56" t="inlineStr">
         <is>
-          <t>A linha JUR-E02B foi criada para receber os encargos e benefícios sobre o salário bruto (INSS patronal, FGTS, provisões de 13º e férias, VT/VR, plano de saúde). Hoje está em branco em mai, jun e jul.</t>
+          <t>A linha JUR-E02B recebe os encargos e benefícios sobre o salário bruto (INSS patronal, FGTS, provisões de 13º e férias, VT/VR, plano de saúde). Hoje está em branco.</t>
         </is>
       </c>
       <c r="D5" s="56" t="inlineStr">
@@ -7909,12 +7909,12 @@
       </c>
       <c r="C6" s="59" t="inlineStr">
         <is>
-          <t>A linha TI-E01B recebe os encargos e benefícios sobre o salário bruto, mesmo tratamento dado à Geovanna. Hoje está em branco. Brutos confirmados pela gestora: R$ 2.570,52 até jul/26 e R$ 3.070,52 a partir de 05/08/26.</t>
+          <t>A linha TI-E01B recebe os encargos e benefícios sobre o salário bruto, mesmo tratamento dado à Geovanna. Hoje está em branco. Brutos confirmados pela gestora: R$ 2.570,52 até jul/26 e R$ 3.070,52 a partir de 05/08/26. O envelope orçado permanece em R$ 5.416,525/mês — o aumento foi absorvido pela folga, não somado ao orçamento.</t>
         </is>
       </c>
       <c r="D6" s="59" t="inlineStr">
         <is>
-          <t>A folga do orçado NÃO é economia estrutural: o custo total de R$ 5.416,53 foi dimensionado prevendo um aumento maior, ainda não concedido. Com o bruto de agosto, a folga praticamente se esgota — a encargos de 67% o custo vai a R$ 5.127,77 (sobram R$ 288,76/mês) e a 80% passa a estourar o orçado. Preencher os encargos reais é o que define se ainda há margem.</t>
+          <t>A folga do orçado NÃO é economia estrutural: o custo total foi dimensionado prevendo um aumento maior, ainda não concedido. Com o bruto de agosto, o orçado de encargos (R$ 2.346,01) equivale a 76% sobre o bruto — dentro da faixa normal (67% a 80%), então pode sobrar ou estourar.</t>
         </is>
       </c>
       <c r="E6" s="59" t="inlineStr">
@@ -7931,22 +7931,22 @@
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="55" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B7" s="56" t="inlineStr">
         <is>
-          <t>Jonathan R$ 3.700/mês abaixo do contratado</t>
+          <t>Reajuste da Thamar — revisão orçamentária</t>
         </is>
       </c>
       <c r="C7" s="56" t="inlineStr">
         <is>
-          <t>Orçado R$ 10.000/mês, realizado R$ 6.300/mês em mai, jun e jul.</t>
+          <t>Reajuste permanente de R$ 5.000 para R$ 5.500/mês, em vigor desde mai/26. O planejado foi mantido em R$ 5.000 nos meses já realizados (para o desvio ficar visível) e revisado para R$ 5.500 de out a dez.</t>
         </is>
       </c>
       <c r="D7" s="56" t="inlineStr">
         <is>
-          <t>Maior desvio em reais de todo o orçamento: R$ 11.100 em três meses. Se o valor menor for o novo padrão, o planejado de ago a dez deve ser revisado para baixo — sobrariam R$ 18.500 no orçamento do TI.</t>
+          <t>Desvio já incorrido de R$ 500/mês. Ao contrário do aumento do Vinicius, este estourou o orçado: não havia folga na linha dela.</t>
         </is>
       </c>
       <c r="E7" s="56" t="inlineStr">
@@ -7956,29 +7956,29 @@
       </c>
       <c r="F7" s="60" t="inlineStr">
         <is>
-          <t>EM ABERTO</t>
+          <t>APLICADO</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="58" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B8" s="59" t="inlineStr">
         <is>
-          <t>Elias Benedito zerado nos três meses</t>
+          <t>Jusbrasil 30% acima do orçado</t>
         </is>
       </c>
       <c r="C8" s="59" t="inlineStr">
         <is>
-          <t>Orçado R$ 1.065/mês como suporte técnico terceirizado, realizado R$ 0 em mai, jun e jul.</t>
+          <t>Orçado R$ 104,90/mês, realizado R$ 136,00/mês em mai, jun e jul.</t>
         </is>
       </c>
       <c r="D8" s="59" t="inlineStr">
         <is>
-          <t>Confirmar se o contrato segue ativo (acionamento sob demanda) ou se foi encerrado. Se encerrado, são R$ 8.520 a liberar no orçamento do ano.</t>
+          <t>Menor desvio em reais (R$ 31,10/mês), mas o maior em percentual. Vale conferir se houve reajuste contratual ou mudança de plano.</t>
         </is>
       </c>
       <c r="E8" s="59" t="inlineStr">
@@ -7986,7 +7986,7 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F8" s="60" t="inlineStr">
+      <c r="F8" s="61" t="inlineStr">
         <is>
           <t>EM ABERTO</t>
         </is>
@@ -7995,22 +7995,22 @@
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="55" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="B9" s="56" t="inlineStr">
         <is>
-          <t>Reajuste da Thamar — revisão orçamentária</t>
+          <t>Bonificação de ago/26 do Jurídico</t>
         </is>
       </c>
       <c r="C9" s="56" t="inlineStr">
         <is>
-          <t>Reajuste permanente de R$ 5.000 para R$ 5.500/mês, já em vigor desde mai/26. O planejado foi mantido em R$ 5.000 em mai–set (para o desvio ficar visível) e revisado para R$ 5.500 de out a dez.</t>
+          <t>Estão orçados R$ 10.293,60 em agosto e R$ 12.867,00 em dezembro. O realizado de agosto ainda não foi informado.</t>
         </is>
       </c>
       <c r="D9" s="56" t="inlineStr">
         <is>
-          <t>Desvio já incorrido de R$ 500/mês. Impacto de +R$ 1.500 no orçamento do restante do ano; o orçamento total sobe para R$ 395.852,68.</t>
+          <t>É a maior despesa isolada do Jurídico no segundo semestre.</t>
         </is>
       </c>
       <c r="E9" s="56" t="inlineStr">
@@ -8020,29 +8020,29 @@
       </c>
       <c r="F9" s="61" t="inlineStr">
         <is>
-          <t>APLICADO</t>
+          <t>EM ABERTO</t>
         </is>
       </c>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="58" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B10" s="59" t="inlineStr">
         <is>
-          <t>Jusbrasil 30% acima do orçado</t>
+          <t>Jonathan R$ 3.700/mês abaixo do contratado</t>
         </is>
       </c>
       <c r="C10" s="59" t="inlineStr">
         <is>
-          <t>Orçado R$ 104,90/mês, realizado R$ 136,00/mês nos três meses.</t>
+          <t>Orçado R$ 10.000/mês, realizado R$ 6.300/mês em mai, jun e jul.</t>
         </is>
       </c>
       <c r="D10" s="59" t="inlineStr">
         <is>
-          <t>Menor desvio em reais (R$ 31,10/mês), mas o maior em percentual. Vale conferir se houve reajuste contratual ou mudança de plano.</t>
+          <t>Maior desvio em reais de todo o orçamento: R$ 11.100 em três meses. Se o valor menor for o novo padrão, o planejado de ago a dez deve ser revisado para baixo — sobrariam R$ 18.500 no orçamento do TI.</t>
         </is>
       </c>
       <c r="E10" s="59" t="inlineStr">
@@ -8050,7 +8050,7 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F10" s="60" t="inlineStr">
+      <c r="F10" s="61" t="inlineStr">
         <is>
           <t>EM ABERTO</t>
         </is>
@@ -8059,22 +8059,22 @@
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="55" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="B11" s="56" t="inlineStr">
         <is>
-          <t>Bonificação de ago/26 do Jurídico</t>
+          <t>Elias Benedito zerado nos três meses</t>
         </is>
       </c>
       <c r="C11" s="56" t="inlineStr">
         <is>
-          <t>Estão orçados R$ 10.293,60 em agosto e R$ 12.867,00 em dezembro. O realizado de agosto ainda não foi informado.</t>
+          <t>Orçado R$ 1.065/mês como suporte técnico terceirizado, realizado R$ 0 em mai, jun e jul.</t>
         </is>
       </c>
       <c r="D11" s="56" t="inlineStr">
         <is>
-          <t>É a maior despesa isolada do Jurídico no segundo semestre. Sem confirmação, o acumulado de agosto fica distorcido.</t>
+          <t>Confirmar se o contrato segue ativo (acionamento sob demanda) ou se foi encerrado. Se encerrado, são R$ 12.780 a liberar no orçamento do ano.</t>
         </is>
       </c>
       <c r="E11" s="56" t="inlineStr">
@@ -8082,7 +8082,7 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F11" s="60" t="inlineStr">
+      <c r="F11" s="61" t="inlineStr">
         <is>
           <t>EM ABERTO</t>
         </is>
@@ -8091,22 +8091,22 @@
     <row r="12" ht="58" customHeight="1">
       <c r="A12" s="58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>H</t>
         </is>
       </c>
       <c r="B12" s="59" t="inlineStr">
         <is>
-          <t>Base de meses — reconciliada com a ficha original</t>
+          <t>Planejado de jan a abr — CONFERIR</t>
         </is>
       </c>
       <c r="C12" s="59" t="inlineStr">
         <is>
-          <t>A ficha trazia a coluna TOTAL do TI digitada à mão em bases diferentes por pessoa (Vinicius e Elias em 12 meses, Jonathan em 9) enquanto o grid mensal tinha só 8 colunas. Com o período estendido para jan–dez, os três totais batem exatamente: R$ 64.998,30 + R$ 12.780,00 + R$ 90.000,00 = R$ 167.778,30, o valor original da ficha. Não era erro de digitação — era o grid que estava incompleto.</t>
+          <t>O 1º quadrimestre foi preenchido replicando os valores mensais conhecidos, porque a ficha original só trazia o grid de mai a dez. Exceções tratadas: Jonathan começa em abr, Thamar a R$ 5.000 (pré-reajuste), Vinicius com bruto de R$ 2.570,52 e Adapta a R$ 1.300 (valor até jun).</t>
         </is>
       </c>
       <c r="D12" s="59" t="inlineStr">
         <is>
-          <t>Equipe de TI volta ao valor original de R$ 167.778,30. Jonathan lançado com entrada em abr/26 (9 meses), que é o que explica os R$ 90.000 da ficha.</t>
+          <t>Se algum contrato tinha valor diferente no 1º quadrimestre, ou se houve bonificação nesse período, o planejado de jan a abr precisa ser corrigido antes de comparar com o realizado.</t>
         </is>
       </c>
       <c r="E12" s="59" t="inlineStr">
@@ -8114,31 +8114,31 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F12" s="61" t="inlineStr">
-        <is>
-          <t>RESOLVIDO</t>
+      <c r="F12" s="62" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
         </is>
       </c>
     </row>
     <row r="13" ht="58" customHeight="1">
       <c r="A13" s="55" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>I</t>
         </is>
       </c>
       <c r="B13" s="56" t="inlineStr">
         <is>
-          <t>Planejado de jan a abr — CONFERIR</t>
+          <t>Realizado de jan a abr — A LANÇAR</t>
         </is>
       </c>
       <c r="C13" s="56" t="inlineStr">
         <is>
-          <t>O 1º quadrimestre foi preenchido replicando os valores mensais já conhecidos, porque a ficha original só trazia o grid de mai a dez. Exceções tratadas: Jonathan começa em abr, Thamar a R$ 5.000 (pré-reajuste), Vinicius com bruto de R$ 2.570,52 e Adapta a R$ 1.300 (valor até jun).</t>
+          <t>As colunas de jan a abr estão em branco na aba Realizado. Só mai, jun e jul foram informados.</t>
         </is>
       </c>
       <c r="D13" s="56" t="inlineStr">
         <is>
-          <t>Se algum contrato tinha valor diferente no 1º quadrimestre, ou se houve bonificação nesse período, o planejado de jan a abr precisa ser corrigido antes de comparar com o realizado.</t>
+          <t>São 4 dos 7 meses já fechados do ano. Sem eles o acumulado e o Painel refletem menos da metade do período decorrido.</t>
         </is>
       </c>
       <c r="E13" s="56" t="inlineStr">
@@ -8146,31 +8146,31 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F13" s="62" t="inlineStr">
-        <is>
-          <t>CONFERIR</t>
+      <c r="F13" s="57" t="inlineStr">
+        <is>
+          <t>A LANÇAR</t>
         </is>
       </c>
     </row>
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="58" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>J</t>
         </is>
       </c>
       <c r="B14" s="59" t="inlineStr">
         <is>
-          <t>Realizado de jan a abr — A LANÇAR</t>
+          <t>Despesas do TI — A LANÇAR</t>
         </is>
       </c>
       <c r="C14" s="59" t="inlineStr">
         <is>
-          <t>As colunas de jan a abr estão em branco na aba Realizado. Só mai, jun e jul foram informados.</t>
+          <t>As 9 linhas de despesas do TI (peças, backup, Adapta, antivírus, Office, sala de reunião, cursos, app de gravação e bonificação) não têm lançamento em nenhum mês.</t>
         </is>
       </c>
       <c r="D14" s="59" t="inlineStr">
         <is>
-          <t>São 4 dos 7 meses já fechados do ano. Sem eles o acumulado e o Painel refletem menos da metade do período decorrido.</t>
+          <t>São R$ 89.040 orçados no ano, 35% do orçamento do TI. Sem lançamento, o departamento aparece com desvio negativo que é ausência de dado.</t>
         </is>
       </c>
       <c r="E14" s="59" t="inlineStr">
@@ -8187,126 +8187,126 @@
     <row r="15" ht="58" customHeight="1">
       <c r="A15" s="55" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B15" s="56" t="inlineStr">
         <is>
-          <t>Origem do valor realizado</t>
+          <t>Base de meses — reconciliada com a ficha original</t>
         </is>
       </c>
       <c r="C15" s="56" t="inlineStr">
         <is>
-          <t>Ainda não definido se o realizado virá de lançamento manual, de relatório do financeiro/ERP por centro de custo, ou misto.</t>
+          <t>A ficha trazia a coluna TOTAL do TI digitada à mão em bases diferentes por pessoa (Vinicius e Elias em 12 meses, Jonathan em 9) enquanto o grid mensal tinha só 8 colunas. Com o período em jan–dez os três totais batem exatamente: R$ 64.998,30 + R$ 12.780,00 + R$ 90.000,00 = R$ 167.778,30, o valor da ficha. Não era erro de digitação — era o grid que estava incompleto.</t>
         </is>
       </c>
       <c r="D15" s="56" t="inlineStr">
         <is>
-          <t>Sem fonte definida o realizado pode divergir da contabilidade e o comparativo perde valor na apresentação à diretoria.</t>
+          <t>Equipe de TI no valor original de R$ 167.778,30. Jonathan lançado com entrada em abr/26 (9 meses), que é o que explica os R$ 90.000.</t>
         </is>
       </c>
       <c r="E15" s="56" t="inlineStr">
         <is>
-          <t>Cristiane + Financeiro</t>
+          <t>Cristiane</t>
         </is>
       </c>
       <c r="F15" s="60" t="inlineStr">
         <is>
-          <t>EM ABERTO</t>
+          <t>RESOLVIDO</t>
         </is>
       </c>
     </row>
     <row r="16" ht="58" customHeight="1">
       <c r="A16" s="58" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B16" s="59" t="inlineStr">
         <is>
-          <t>Jusfy x Astrea</t>
+          <t>Origem do valor realizado</t>
         </is>
       </c>
       <c r="C16" s="59" t="inlineStr">
         <is>
-          <t>O risco era pagar os dois em paralelo. O realizado de mai–jul mostra Astrea em R$ 0 (cancelado) e Jusfy em R$ 0 (ainda não iniciado) — no momento não há custo de nenhum dos dois.</t>
+          <t>Ainda não definido se o realizado virá de lançamento manual, de relatório do financeiro/ERP por centro de custo, ou misto. Até aqui os números vieram informados pela gestora.</t>
         </is>
       </c>
       <c r="D16" s="59" t="inlineStr">
         <is>
-          <t>Economia de R$ 212,07/mês enquanto durar. Falta decidir se o Jusfy entra e quando, para ajustar o planejado de ago a dez.</t>
+          <t>Sem fonte definida o realizado pode divergir da contabilidade e o comparativo perde valor na apresentação à diretoria.</t>
         </is>
       </c>
       <c r="E16" s="59" t="inlineStr">
         <is>
-          <t>Cristiane</t>
+          <t>Cristiane + Financeiro</t>
         </is>
       </c>
       <c r="F16" s="61" t="inlineStr">
         <is>
-          <t>RESOLVIDO</t>
+          <t>EM ABERTO</t>
         </is>
       </c>
     </row>
     <row r="17" ht="58" customHeight="1">
       <c r="A17" s="55" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B17" s="56" t="inlineStr">
         <is>
-          <t>Rateio dos softwares corporativos de TI</t>
+          <t>Jusfy x Astrea</t>
         </is>
       </c>
       <c r="C17" s="56" t="inlineStr">
         <is>
-          <t>Backup (R$ 6.600), Adapta/IA (R$ 12.200), Antivírus (R$ 1.920) e Office 365 (R$ 3.000) estão marcados na ficha como 'não sei se seria administrativo'. Total: R$ 23.720.</t>
+          <t>O risco era pagar os dois em paralelo. O realizado de mai–jul mostra Astrea em R$ 0 (cancelado) e Jusfy em R$ 0 (ainda não iniciado) — no momento não há custo de nenhum dos dois.</t>
         </is>
       </c>
       <c r="D17" s="56" t="inlineStr">
         <is>
-          <t>Se são da empresa toda e ficam no centro de custo de TI, o TI carrega despesa que não é dele e aparece caro no comparativo.</t>
+          <t>Economia de R$ 212,07/mês enquanto durar. Falta decidir se o Jusfy entra e quando, para ajustar o planejado dos meses seguintes.</t>
         </is>
       </c>
       <c r="E17" s="56" t="inlineStr">
         <is>
-          <t>Cristiane + Controladoria</t>
+          <t>Cristiane</t>
         </is>
       </c>
       <c r="F17" s="60" t="inlineStr">
         <is>
-          <t>EM ABERTO</t>
+          <t>RESOLVIDO</t>
         </is>
       </c>
     </row>
     <row r="18" ht="58" customHeight="1">
       <c r="A18" s="58" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B18" s="59" t="inlineStr">
         <is>
-          <t>Sala de Reunião — recorrente ou pontual?</t>
+          <t>Rateio dos softwares corporativos de TI</t>
         </is>
       </c>
       <c r="C18" s="59" t="inlineStr">
         <is>
-          <t>R$ 2.800/mês × 8 = R$ 22.400 diluídos linearmente, classificados em Móveis e Utensílios.</t>
+          <t>Backup (R$ 9.900), Adapta/IA (R$ 17.400), Antivírus (R$ 2.880) e Office 365 (R$ 4.500) estão marcados na ficha como 'não sei se seria administrativo'. Total no ano: R$ 34.680.</t>
         </is>
       </c>
       <c r="D18" s="59" t="inlineStr">
         <is>
-          <t>Se for compra pontual (CAPEX), o desvio mensal vai acusar alarme falso todo mês até a compra acontecer, e um pico no mês da compra.</t>
+          <t>São 39% das despesas do TI. Se são da empresa toda e ficam no centro de custo de TI, o departamento carrega despesa que não é dele e aparece caro.</t>
         </is>
       </c>
       <c r="E18" s="59" t="inlineStr">
         <is>
-          <t>Cristiane</t>
-        </is>
-      </c>
-      <c r="F18" s="60" t="inlineStr">
+          <t>Cristiane + Controladoria</t>
+        </is>
+      </c>
+      <c r="F18" s="61" t="inlineStr">
         <is>
           <t>EM ABERTO</t>
         </is>
@@ -8315,22 +8315,22 @@
     <row r="19" ht="58" customHeight="1">
       <c r="A19" s="55" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B19" s="56" t="inlineStr">
         <is>
-          <t>Office 365 — nº de licenças</t>
+          <t>Sala de Reunião — recorrente ou pontual?</t>
         </is>
       </c>
       <c r="C19" s="56" t="inlineStr">
         <is>
-          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+          <t>R$ 2.800/mês × 12 = R$ 33.600 diluídos linearmente, classificados em Móveis e Utensílios.</t>
         </is>
       </c>
       <c r="D19" s="56" t="inlineStr">
         <is>
-          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+          <t>Se for compra pontual (CAPEX), o desvio mensal vai acusar alarme falso todo mês até a compra acontecer, e um pico no mês da compra.</t>
         </is>
       </c>
       <c r="E19" s="56" t="inlineStr">
@@ -8338,7 +8338,7 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F19" s="60" t="inlineStr">
+      <c r="F19" s="61" t="inlineStr">
         <is>
           <t>EM ABERTO</t>
         </is>
@@ -8347,30 +8347,62 @@
     <row r="20" ht="58" customHeight="1">
       <c r="A20" s="58" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B20" s="59" t="inlineStr">
+        <is>
+          <t>Office 365 — nº de licenças</t>
+        </is>
+      </c>
+      <c r="C20" s="59" t="inlineStr">
+        <is>
+          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+        </is>
+      </c>
+      <c r="D20" s="59" t="inlineStr">
+        <is>
+          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+        </is>
+      </c>
+      <c r="E20" s="59" t="inlineStr">
+        <is>
+          <t>Cristiane</t>
+        </is>
+      </c>
+      <c r="F20" s="61" t="inlineStr">
+        <is>
+          <t>EM ABERTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="55" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B20" s="59" t="inlineStr">
+      <c r="B21" s="56" t="inlineStr">
         <is>
           <t>Critério de competência x caixa</t>
         </is>
       </c>
-      <c r="C20" s="59" t="inlineStr">
+      <c r="C21" s="56" t="inlineStr">
         <is>
           <t>Definir se o realizado será lançado pela data de pagamento (caixa) ou pelo mês de referência da despesa (competência).</t>
         </is>
       </c>
-      <c r="D20" s="59" t="inlineStr">
+      <c r="D21" s="56" t="inlineStr">
         <is>
           <t>Misturar os dois critérios gera desvio artificial em meses de virada, principalmente em folha e prêmios.</t>
         </is>
       </c>
-      <c r="E20" s="59" t="inlineStr">
+      <c r="E21" s="56" t="inlineStr">
         <is>
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F20" s="60" t="inlineStr">
+      <c r="F21" s="61" t="inlineStr">
         <is>
           <t>EM ABERTO</t>
         </is>

</xml_diff>

<commit_message>
feat(orcamento): IAs marcadas para rateio
Claude, GPT, Adapta One e Adapta Skip recebem "RATEIO A DEFINIR", como
ja tinham Backup, Adapta, Antivirus e Office 365 — oito linhas de uso
transversal ao todo.

O extrato mostra que o rateio ja acontece sem regra: a OpenAI
(R$ 5.950,10) caiu no centro de custo do TI e o Adapta (R$ 3.351) no
Juridico, mesma natureza de gasto em centros diferentes por acaso.

Pendencias L e 4 reescritas para tratar softwares corporativos e IAs
sob o mesmo criterio, com a sugestao de manter o contrato centralizado
no TI e ratear por usuario ativo, metrica que as plataformas fornecem.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -24647,7 +24647,7 @@
       </c>
       <c r="E26" s="48" t="inlineStr">
         <is>
-          <t>Ferramenta de IA — não constava na ficha. Planejado a definir com a diretoria</t>
+          <t>Ferramenta de IA — não constava na ficha. Planejado a definir com a diretoria. RATEIO A DEFINIR: uso transversal entre as áreas</t>
         </is>
       </c>
       <c r="F26" s="47" t="inlineStr"/>
@@ -24720,7 +24720,7 @@
       </c>
       <c r="E27" s="48" t="inlineStr">
         <is>
-          <t>Ferramenta de IA — não constava na ficha. Planejado a definir com a diretoria</t>
+          <t>Ferramenta de IA — não constava na ficha. Planejado a definir com a diretoria. RATEIO A DEFINIR: uso transversal entre as áreas</t>
         </is>
       </c>
       <c r="F27" s="47" t="inlineStr"/>
@@ -24793,7 +24793,7 @@
       </c>
       <c r="E28" s="48" t="inlineStr">
         <is>
-          <t>Ferramenta de IA — não constava na ficha. Planejado a definir com a diretoria. CONFERIR sobreposição com a linha 'Inteligência Artificial (Adapta)'</t>
+          <t>Ferramenta de IA — não constava na ficha. Planejado a definir com a diretoria. RATEIO A DEFINIR: uso transversal entre as áreas. CONFERIR sobreposição com a linha 'Inteligência Artificial (Adapta)'</t>
         </is>
       </c>
       <c r="F28" s="47" t="inlineStr"/>
@@ -24866,7 +24866,7 @@
       </c>
       <c r="E29" s="48" t="inlineStr">
         <is>
-          <t>Ferramenta de IA — não constava na ficha. Planejado a definir com a diretoria. CONFERIR o nome exato do produto e a sobreposição com 'Inteligência Artificial (Adapta)'</t>
+          <t>Ferramenta de IA — não constava na ficha. Planejado a definir com a diretoria. RATEIO A DEFINIR: uso transversal entre as áreas. CONFERIR o nome exato do produto e a sobreposição com 'Inteligência Artificial (Adapta)'</t>
         </is>
       </c>
       <c r="F29" s="47" t="inlineStr"/>
@@ -28586,17 +28586,17 @@
       </c>
       <c r="B23" s="69" t="inlineStr">
         <is>
-          <t>Ferramentas de IA sem orçamento — DEFINIR META</t>
+          <t>Ferramentas de IA — DEFINIR META E RATEIO</t>
         </is>
       </c>
       <c r="C23" s="69" t="inlineStr">
         <is>
-          <t>Claude, GPT, Adapta One e Adapta Skip são gastos que existem hoje e não constavam na ficha. Foram criadas quatro linhas separadas, com planejado zerado, para a meta ser definida junto com a diretoria.</t>
+          <t>Claude, GPT, Adapta One e Adapta Skip existem hoje e não constavam na ficha. Quatro linhas criadas com planejado zerado, à espera da meta. Todas marcadas com RATEIO A DEFINIR: são de uso transversal, não exclusivo do TI.</t>
         </is>
       </c>
       <c r="D23" s="69" t="inlineStr">
         <is>
-          <t>Enquanto o planejado for zero, qualquer lançamento nessas linhas aparece como 'Não orçado'. Conferir também se há sobreposição com a linha 'Inteligência Artificial (Adapta)', já orçada em R$ 17.400/ano — pode ser que ela já cubra o Adapta One e o Adapta Skip. E confirmar o nome exato do 'Adapta Skip'.</t>
+          <t>O rateio já acontece de fato, mas sem regra: no extrato, a OpenAI (R$ 5.950,10) caiu no centro de custo do TI e o Adapta (R$ 3.351) caiu no Jurídico — mesma natureza de gasto, centros diferentes por acaso. Sem critério definido, o TI absorve custo de ferramenta que a empresa inteira usa e aparece caro na comparação, enquanto as áreas usuárias não enxergam o que consomem. Sugestão: manter o contrato centralizado no TI (facilita negociação e controle de licenças) e ratear o custo por usuário ativo, que é métrica que as próprias plataformas fornecem. Conferir também a sobreposição com 'Inteligência Artificial (Adapta)', já orçada em R$ 17.400/ano, e o nome exato do 'Adapta Skip'.</t>
         </is>
       </c>
       <c r="E23" s="69" t="inlineStr">
@@ -28618,17 +28618,17 @@
       </c>
       <c r="B24" s="72" t="inlineStr">
         <is>
-          <t>Rateio dos softwares corporativos de TI</t>
+          <t>Rateio dos softwares corporativos e das IAs</t>
         </is>
       </c>
       <c r="C24" s="72" t="inlineStr">
         <is>
-          <t>Backup (R$ 9.900), Adapta/IA (R$ 17.400), Antivírus (R$ 2.880) e Office 365 (R$ 4.500) estão marcados na ficha como 'não sei se seria administrativo'. Total no ano: R$ 34.680.</t>
+          <t>Backup (R$ 9.900), Adapta/IA (R$ 17.400), Antivírus (R$ 2.880) e Office 365 (R$ 4.500) estão marcados na ficha como 'não sei se seria administrativo' — R$ 34.680 no ano. Somam-se a eles as quatro ferramentas de IA do item L, também de uso transversal.</t>
         </is>
       </c>
       <c r="D24" s="72" t="inlineStr">
         <is>
-          <t>São 39% das despesas do TI. Se são da empresa toda e ficam no centro de custo de TI, o departamento carrega despesa que não é dele e aparece caro.</t>
+          <t>São 39% das despesas orçadas do TI, mais o que vier das IAs. Se são da empresa toda e ficam no centro de custo de TI, o departamento carrega despesa que não é dele e aparece caro. Tratar os dois blocos com o mesmo critério de rateio, para não criar duas regras diferentes.</t>
         </is>
       </c>
       <c r="E24" s="72" t="inlineStr">

</xml_diff>

<commit_message>
feat(orcamento): sala de reuniao vira decisao de executar, pausar ou repensar
A pendencia 5 tratava so do formato do lancamento (recorrente x
pontual). Passa a tratar a decisao de fundo levantada pela gestora: a
sala ja nao comporta todas as pessoas, entao investir na configuracao
atual pode nao resolver o problema.

Sao R$ 33.600 no ano, a maior despesa isolada do TI e 38% do que a area
tem orcado em despesas, sem nenhum lancamento ate jul/26. Pausar
liberaria mais que a economia atual do departamento. A questao do
CAPEX pontual x diluido continua registrada, condicionada a decisao de
executar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -28682,27 +28682,27 @@
       </c>
       <c r="B26" s="72" t="inlineStr">
         <is>
-          <t>Sala de Reunião — recorrente ou pontual?</t>
+          <t>Sala de Reunião — EXECUTAR, PAUSAR OU REPENSAR?</t>
         </is>
       </c>
       <c r="C26" s="72" t="inlineStr">
         <is>
-          <t>R$ 2.800/mês × 12 = R$ 33.600 diluídos linearmente, classificados em Móveis e Utensílios.</t>
+          <t>Projeto orçado em R$ 2.800/mês × 12 = R$ 33.600, classificado em Móveis e Utensílios, sem nenhum lançamento até jul/26. A gestora levanta que a sala já não comporta todas as pessoas, então investir na configuração atual pode não resolver o problema real. Três caminhos: executar como está, pausar, ou repensar a solução (outro espaço, formato híbrido, mais de uma sala).</t>
         </is>
       </c>
       <c r="D26" s="72" t="inlineStr">
         <is>
-          <t>Se for compra pontual (CAPEX), o desvio mensal vai acusar alarme falso todo mês até a compra acontecer, e um pico no mês da compra.</t>
+          <t>É a maior despesa isolada do TI e 38% de tudo que a área tem orçado em despesas. Se pausar, são R$ 33.600 liberados — mais que a economia atual do departamento. Decidir antes de comprometer o valor. Se a decisão for executar, definir também se é compra pontual ou parcelada: hoje está diluída linearmente, e se for compra única o desvio mensal vai acusar economia falsa todo mês até a compra e um pico no mês em que ocorrer.</t>
         </is>
       </c>
       <c r="E26" s="72" t="inlineStr">
         <is>
-          <t>Cristiane</t>
-        </is>
-      </c>
-      <c r="F26" s="74" t="inlineStr">
-        <is>
-          <t>EM ABERTO</t>
+          <t>Cristiane + Diretoria</t>
+        </is>
+      </c>
+      <c r="F26" s="75" t="inlineStr">
+        <is>
+          <t>PAUTA REUNIÃO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(orcamento): pendencia de governanca dos notebooks
Cada area tem a propria linha de orcamento para notebooks, mas e o TI
que recebe a solicitacao e executa a compra. Sem acompanhamento do
saldo das outras areas, o TI aprova pedidos sem saber quanto resta em
cada uma e acaba executando um estouro que nao e dele — descoberto so
no fechamento.

Nova pendencia R: o TI passa a acompanhar o saldo da rubrica de
notebooks por area e avisa antes de comprar quando a solicitacao levar
ao estouro. Com o centro de custo no SIENGE o acompanhamento sai do
mesmo relatorio. Fica para a diretoria definir quem da o aval quando o
saldo acabar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -27945,7 +27945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -28709,62 +28709,94 @@
     <row r="27" ht="58" customHeight="1">
       <c r="A27" s="68" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>R</t>
         </is>
       </c>
       <c r="B27" s="69" t="inlineStr">
         <is>
-          <t>Office 365 — nº de licenças</t>
+          <t>Notebooks — TI compra, mas não enxerga o saldo das áreas</t>
         </is>
       </c>
       <c r="C27" s="69" t="inlineStr">
         <is>
-          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+          <t>Cada área tem a própria linha de orçamento para notebooks, mas é o TI que recebe a solicitação e executa a compra quando surge a necessidade. Hoje o TI não tem acompanhamento do orçamento das outras áreas, então aprova pedidos sem saber quanto resta em cada uma.</t>
         </is>
       </c>
       <c r="D27" s="69" t="inlineStr">
         <is>
-          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+          <t>O TI vira o executor de um estouro que não é dele e que ninguém percebe antes de acontecer — a área descobre no fechamento, quando já comprou. Proposta: o TI passa a acompanhar o saldo da rubrica de notebooks de cada área e avisa quando a solicitação for levar ao estouro, antes de comprar. Com o centro de custo no SIENGE, esse acompanhamento sai do mesmo relatório. Definir com a diretoria quem dá o aval quando o saldo acabar: a área solicitante, o TI ou a controladoria.</t>
         </is>
       </c>
       <c r="E27" s="69" t="inlineStr">
         <is>
-          <t>Cristiane</t>
-        </is>
-      </c>
-      <c r="F27" s="74" t="inlineStr">
-        <is>
-          <t>EM ABERTO</t>
+          <t>Cristiane + Diretoria</t>
+        </is>
+      </c>
+      <c r="F27" s="75" t="inlineStr">
+        <is>
+          <t>PAUTA REUNIÃO</t>
         </is>
       </c>
     </row>
     <row r="28" ht="58" customHeight="1">
       <c r="A28" s="71" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B28" s="72" t="inlineStr">
+        <is>
+          <t>Office 365 — nº de licenças</t>
+        </is>
+      </c>
+      <c r="C28" s="72" t="inlineStr">
+        <is>
+          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+        </is>
+      </c>
+      <c r="D28" s="72" t="inlineStr">
+        <is>
+          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+        </is>
+      </c>
+      <c r="E28" s="72" t="inlineStr">
+        <is>
+          <t>Cristiane</t>
+        </is>
+      </c>
+      <c r="F28" s="74" t="inlineStr">
+        <is>
+          <t>EM ABERTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="58" customHeight="1">
+      <c r="A29" s="68" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B28" s="72" t="inlineStr">
+      <c r="B29" s="69" t="inlineStr">
         <is>
           <t>Competência x caixa — DECIDIR O REGIME</t>
         </is>
       </c>
-      <c r="C28" s="72" t="inlineStr">
+      <c r="C29" s="69" t="inlineStr">
         <is>
           <t>Confirmado pela gestora: TODOS os PJs das duas áreas prestam o serviço e recebem no mês seguinte — no Jurídico, Miguel, Thamar e Dra. Michele; no TI, Elias e Jonathan. O que foi pago em jan/26 é serviço de dez/2025, e o serviço de dez/26 só será pago em jan/2027. Hoje o realizado está lançado por CAIXA (mês do pagamento), que é como os valores foram informados, enquanto o orçamento foi montado por COMPETÊNCIA (mês do serviço). São bases diferentes no mesmo comparativo.</t>
         </is>
       </c>
-      <c r="D28" s="72" t="inlineStr">
+      <c r="D29" s="69" t="inlineStr">
         <is>
           <t>RECOMENDAÇÃO: migrar para competência, deslocando os PJs um mês para trás. Motivos: (1) o orçamento já é de competência, então acaba a comparação de bases diferentes; (2) por caixa, o ano de 2026 carrega um mês de 2025 e perde dez/26, o que distorce sempre que o valor muda no meio do ano — no Miguel, R$ 47.250 por caixa contra R$ 49.318 por competência em jan–jul, R$ 2.068 de diferença; (3) o SIENGE gera os dois regimes, então é escolha de configuração. Contra: caixa é mais fácil de bater com o extrato bancário. Decidir UMA vez e manter, senão o histórico mistura critérios. ATENÇÃO NO JONATHAN: o planejado dele começa em abr/26 (competência) e o realizado também foi lançado a partir de abr (caixa) — se ele recebe no mês seguinte, o pagamento de abril é serviço de março, e ou a entrada dele foi em março, ou o realizado de abril deveria ser zero. Conferir junto com a decisão do regime.</t>
         </is>
       </c>
-      <c r="E28" s="72" t="inlineStr">
+      <c r="E29" s="69" t="inlineStr">
         <is>
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F28" s="76" t="inlineStr">
+      <c r="F29" s="76" t="inlineStr">
         <is>
           <t>DECIDIR</t>
         </is>

</xml_diff>

<commit_message>
feat(orcamento): recomendacao sobre papelaria e separacao da sala de reuniao
Pendencia U: papelaria deve ficar no Administrativo, nao no TI. O TI
controla equipamento porque ha decisao tecnica envolvida; em caneta e
bloco nao ha. A troca 1x1 nao se aplica (papelaria acaba, nao quebra),
nao ha patrimonio para rastrear e o custo de controlar o item supera o
item. Se estiver caindo no TI por motivo historico, e o mesmo caso do
Adapta: corrigir na origem.

A pendencia 5 ganha a observacao de que a descricao do projeto da sala
mistura infraestrutura de reuniao (cameras, microfones, cadeiras) com
material de consumo e brindes (canetas, blocos personalizados, copos),
que sao papelaria e pertencem ao Administrativo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -28287,7 +28287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -29034,7 +29034,7 @@
       </c>
       <c r="D26" s="72" t="inlineStr">
         <is>
-          <t>É a maior despesa isolada do TI e 38% de tudo que a área tem orçado em despesas. Se pausar, são R$ 33.600 liberados — mais que a economia atual do departamento. Decidir antes de comprometer o valor. Se a decisão for executar, definir também se é compra pontual ou parcelada: hoje está diluída linearmente, e se for compra única o desvio mensal vai acusar economia falsa todo mês até a compra e um pico no mês em que ocorrer.</t>
+          <t>É a maior despesa isolada do TI e 38% de tudo que a área tem orçado em despesas. Se pausar, são R$ 33.600 liberados — mais que a economia atual do departamento. Decidir antes de comprometer o valor. Se a decisão for executar, definir também se é compra pontual ou parcelada: hoje está diluída linearmente, e se for compra única o desvio mensal vai acusar economia falsa todo mês até a compra e um pico no mês em que ocorrer. SEPARAR OS ITENS: a descrição na ficha mistura infraestrutura de reunião (câmeras, microfones, cadeiras) com material de consumo e brindes (canetas, blocos personalizados, copos, cafeteira). O segundo grupo é papelaria e deveria estar no Administrativo, não no TI (item U).</t>
         </is>
       </c>
       <c r="E26" s="72" t="inlineStr">
@@ -29147,62 +29147,94 @@
     <row r="30" ht="58" customHeight="1">
       <c r="A30" s="71" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B30" s="72" t="inlineStr">
         <is>
-          <t>Office 365 — nº de licenças</t>
+          <t>Papelaria não é TI — manter no Administrativo</t>
         </is>
       </c>
       <c r="C30" s="72" t="inlineStr">
         <is>
-          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+          <t>Recomendação registrada: o controle de papelaria (canetas, blocos, papel, copos) deve ficar no Administrativo/Facilities, não no TI. O TI controla equipamento porque há decisão TÉCNICA envolvida — se o notebook precisa de troca ou só de formatação, se a tela quebrou por defeito ou por queda. Não existe decisão técnica em caneta e bloco.</t>
         </is>
       </c>
       <c r="D30" s="72" t="inlineStr">
         <is>
-          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+          <t>Três diferenças separam as duas coisas: (1) papelaria acaba, não quebra, então a regra de troca 1x1 não se aplica — o controle é de estoque por ponto de pedido, outra lógica; (2) não há patrimônio nem número de série para rastrear item a item; (3) o custo de controlar uma caneta é maior que a caneta. Se papelaria estiver caindo no orçamento do TI por motivo histórico, é o mesmo caso do Adapta (item Q): classificação errada, corrigir na origem quando o centro de custo novo for aberto.</t>
         </is>
       </c>
       <c r="E30" s="72" t="inlineStr">
         <is>
-          <t>Cristiane</t>
+          <t>Cristiane + Administrativo</t>
         </is>
       </c>
       <c r="F30" s="74" t="inlineStr">
         <is>
-          <t>EM ABERTO</t>
+          <t>RECOMENDAÇÃO</t>
         </is>
       </c>
     </row>
     <row r="31" ht="58" customHeight="1">
       <c r="A31" s="68" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B31" s="69" t="inlineStr">
+        <is>
+          <t>Office 365 — nº de licenças</t>
+        </is>
+      </c>
+      <c r="C31" s="69" t="inlineStr">
+        <is>
+          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+        </is>
+      </c>
+      <c r="D31" s="69" t="inlineStr">
+        <is>
+          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+        </is>
+      </c>
+      <c r="E31" s="69" t="inlineStr">
+        <is>
+          <t>Cristiane</t>
+        </is>
+      </c>
+      <c r="F31" s="74" t="inlineStr">
+        <is>
+          <t>EM ABERTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="58" customHeight="1">
+      <c r="A32" s="71" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B31" s="69" t="inlineStr">
+      <c r="B32" s="72" t="inlineStr">
         <is>
           <t>Competência x caixa — DECIDIR O REGIME</t>
         </is>
       </c>
-      <c r="C31" s="69" t="inlineStr">
+      <c r="C32" s="72" t="inlineStr">
         <is>
           <t>Confirmado pela gestora: TODOS os PJs das duas áreas prestam o serviço e recebem no mês seguinte — no Jurídico, Miguel, Thamar e Dra. Michele; no TI, Elias e Jonathan. O que foi pago em jan/26 é serviço de dez/2025, e o serviço de dez/26 só será pago em jan/2027. Hoje o realizado está lançado por CAIXA (mês do pagamento), que é como os valores foram informados, enquanto o orçamento foi montado por COMPETÊNCIA (mês do serviço). São bases diferentes no mesmo comparativo.</t>
         </is>
       </c>
-      <c r="D31" s="69" t="inlineStr">
+      <c r="D32" s="72" t="inlineStr">
         <is>
           <t>RECOMENDAÇÃO: migrar para competência, deslocando os PJs um mês para trás. Motivos: (1) o orçamento já é de competência, então acaba a comparação de bases diferentes; (2) por caixa, o ano de 2026 carrega um mês de 2025 e perde dez/26, o que distorce sempre que o valor muda no meio do ano — no Miguel, R$ 47.250 por caixa contra R$ 49.318 por competência em jan–jul, R$ 2.068 de diferença; (3) o SIENGE gera os dois regimes, então é escolha de configuração. Contra: caixa é mais fácil de bater com o extrato bancário. Decidir UMA vez e manter, senão o histórico mistura critérios. ATENÇÃO NO JONATHAN: o planejado dele começa em abr/26 (competência) e o realizado também foi lançado a partir de abr (caixa) — se ele recebe no mês seguinte, o pagamento de abril é serviço de março, e ou a entrada dele foi em março, ou o realizado de abril deveria ser zero. Conferir junto com a decisão do regime.</t>
         </is>
       </c>
-      <c r="E31" s="69" t="inlineStr">
+      <c r="E32" s="72" t="inlineStr">
         <is>
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F31" s="76" t="inlineStr">
+      <c r="F32" s="76" t="inlineStr">
         <is>
           <t>DECIDIR</t>
         </is>

</xml_diff>

<commit_message>
feat(orcamento): pendencia para confirmar Claude x GPT com a diretoria
Item W: perguntar ao Vitor se ele seguira usando Claude, GPT ou os
dois. As duas ferramentas tem a mesma finalidade, entao manter ambas
para o mesmo usuario e redundancia paga.

E pre-requisito da meta do item L: nao da para dimensionar o orcamento
de IA sem saber quantas licencas de cada ferramenta ficam de pe.
Registrada a referencia de custo da OpenAI no extrato (R$ 5.950,10 em
sete meses, R$ 5.394 so em abril) e a observacao de que o levantamento
deve alcancar todos os usuarios, nao so a diretoria.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -28486,7 +28486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -29410,62 +29410,94 @@
     <row r="32" ht="58" customHeight="1">
       <c r="A32" s="71" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>W</t>
         </is>
       </c>
       <c r="B32" s="72" t="inlineStr">
         <is>
-          <t>Office 365 — nº de licenças</t>
+          <t>Vitor (diretoria) — Claude ou GPT? PERGUNTAR</t>
         </is>
       </c>
       <c r="C32" s="72" t="inlineStr">
         <is>
-          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+          <t>Confirmar com o Vitor se ele seguirá usando o Claude, o GPT, ou os dois. Hoje as duas ferramentas estão contratadas e são de mesma finalidade — IA generalista —, então manter as duas para o mesmo usuário é redundância paga.</t>
         </is>
       </c>
       <c r="D32" s="72" t="inlineStr">
         <is>
-          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+          <t>É pré-requisito para fechar a meta do item L: não dá para dimensionar o orçamento de IA sem saber quantas licenças de cada ferramenta ficam de pé. Referência de custo: a OpenAI aparece no extrato com R$ 5.950,10 em sete meses, sendo R$ 5.394 só em abr/26. Levantar a mesma informação para os demais usuários, não só a diretoria — a decisão vale para todo mundo.</t>
         </is>
       </c>
       <c r="E32" s="72" t="inlineStr">
         <is>
-          <t>Cristiane</t>
+          <t>Cristiane + Vitor</t>
         </is>
       </c>
       <c r="F32" s="74" t="inlineStr">
         <is>
-          <t>EM ABERTO</t>
+          <t>PERGUNTAR</t>
         </is>
       </c>
     </row>
     <row r="33" ht="58" customHeight="1">
       <c r="A33" s="68" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B33" s="69" t="inlineStr">
+        <is>
+          <t>Office 365 — nº de licenças</t>
+        </is>
+      </c>
+      <c r="C33" s="69" t="inlineStr">
+        <is>
+          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+        </is>
+      </c>
+      <c r="D33" s="69" t="inlineStr">
+        <is>
+          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+        </is>
+      </c>
+      <c r="E33" s="69" t="inlineStr">
+        <is>
+          <t>Cristiane</t>
+        </is>
+      </c>
+      <c r="F33" s="74" t="inlineStr">
+        <is>
+          <t>EM ABERTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="58" customHeight="1">
+      <c r="A34" s="71" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B33" s="69" t="inlineStr">
+      <c r="B34" s="72" t="inlineStr">
         <is>
           <t>Competência x caixa — DECIDIR O REGIME</t>
         </is>
       </c>
-      <c r="C33" s="69" t="inlineStr">
+      <c r="C34" s="72" t="inlineStr">
         <is>
           <t>Confirmado pela gestora: TODOS os PJs das duas áreas prestam o serviço e recebem no mês seguinte — no Jurídico, Miguel, Thamar e Dra. Michele; no TI, Elias e Jonathan. O que foi pago em jan/26 é serviço de dez/2025, e o serviço de dez/26 só será pago em jan/2027. Hoje o realizado está lançado por CAIXA (mês do pagamento), que é como os valores foram informados, enquanto o orçamento foi montado por COMPETÊNCIA (mês do serviço). São bases diferentes no mesmo comparativo.</t>
         </is>
       </c>
-      <c r="D33" s="69" t="inlineStr">
+      <c r="D34" s="72" t="inlineStr">
         <is>
           <t>RECOMENDAÇÃO: migrar para competência, deslocando os PJs um mês para trás. Motivos: (1) o orçamento já é de competência, então acaba a comparação de bases diferentes; (2) por caixa, o ano de 2026 carrega um mês de 2025 e perde dez/26, o que distorce sempre que o valor muda no meio do ano — no Miguel, R$ 47.250 por caixa contra R$ 49.318 por competência em jan–jul, R$ 2.068 de diferença; (3) o SIENGE gera os dois regimes, então é escolha de configuração. Contra: caixa é mais fácil de bater com o extrato bancário. Decidir UMA vez e manter, senão o histórico mistura critérios. ATENÇÃO NO JONATHAN: o planejado dele começa em abr/26 (competência) e o realizado também foi lançado a partir de abr (caixa) — se ele recebe no mês seguinte, o pagamento de abril é serviço de março, e ou a entrada dele foi em março, ou o realizado de abril deveria ser zero. Conferir junto com a decisão do regime.</t>
         </is>
       </c>
-      <c r="E33" s="69" t="inlineStr">
+      <c r="E34" s="72" t="inlineStr">
         <is>
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F33" s="76" t="inlineStr">
+      <c r="F34" s="76" t="inlineStr">
         <is>
           <t>DECIDIR</t>
         </is>

</xml_diff>

<commit_message>
feat(orcamento): mapa de licencas de IA e risco de compartilhamento
Item X registra a situacao conhecida: a licenca do GPT era da Thamar e
hoje e usada em conjunto por Gil, Miguel e Thamar, e uma licenca foi
cedida ao Financeiro.

Duas consequencias registradas. Orcamento: licenca usada pelo
Financeiro e custo de outra area lancado no TI/Juridico, exatamente o
que o rateio do item L precisa resolver — e sem o mapa completo nao ha
como ratear. Risco: contas de IA generalista sao individuais e o
compartilhamento costuma contrariar os termos de uso, com risco de
suspensao; num escritorio de advocacia o agravante e o historico de
conversas ficar visivel para todos que usam o mesmo login, expondo
dados de cliente a quem nao atua no caso.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -28486,7 +28486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -29442,62 +29442,94 @@
     <row r="33" ht="58" customHeight="1">
       <c r="A33" s="68" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>X</t>
         </is>
       </c>
       <c r="B33" s="69" t="inlineStr">
         <is>
-          <t>Office 365 — nº de licenças</t>
+          <t>Mapa de licenças de IA — quem usa o quê</t>
         </is>
       </c>
       <c r="C33" s="69" t="inlineStr">
         <is>
-          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+          <t>Situação atual conhecida: a licença do GPT era da Thamar e hoje é usada em conjunto por Gil, Miguel e Thamar. Uma licença também foi cedida ao Financeiro. Falta o mapa completo — quem usa cada ferramenta, em qual área e sob qual login.</t>
         </is>
       </c>
       <c r="D33" s="69" t="inlineStr">
         <is>
-          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+          <t>Duas consequências. ORÇAMENTO: uma licença usada pelo Financeiro é custo de outra área lançado no TI/Jurídico — é exatamente o caso que o rateio do item L precisa resolver, e sem o mapa não há como ratear. RISCO: contas de IA generalista são individuais, e o compartilhamento entre pessoas costuma contrariar os termos de uso do fornecedor, com risco de suspensão. Mais grave num escritório de advocacia: o histórico de conversas fica visível para todos que usam o mesmo login, então dados de um cliente podem ser vistos por quem não atua no caso — questão de sigilo profissional, não só de custo. Avaliar licenças individuais ou plano de equipe, que costuma sair mais barato por usuário e separa os históricos.</t>
         </is>
       </c>
       <c r="E33" s="69" t="inlineStr">
         <is>
-          <t>Cristiane</t>
+          <t>Cristiane + Vitor</t>
         </is>
       </c>
       <c r="F33" s="74" t="inlineStr">
         <is>
-          <t>EM ABERTO</t>
+          <t>LEVANTAR</t>
         </is>
       </c>
     </row>
     <row r="34" ht="58" customHeight="1">
       <c r="A34" s="71" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B34" s="72" t="inlineStr">
+        <is>
+          <t>Office 365 — nº de licenças</t>
+        </is>
+      </c>
+      <c r="C34" s="72" t="inlineStr">
+        <is>
+          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+        </is>
+      </c>
+      <c r="D34" s="72" t="inlineStr">
+        <is>
+          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+        </is>
+      </c>
+      <c r="E34" s="72" t="inlineStr">
+        <is>
+          <t>Cristiane</t>
+        </is>
+      </c>
+      <c r="F34" s="74" t="inlineStr">
+        <is>
+          <t>EM ABERTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="58" customHeight="1">
+      <c r="A35" s="68" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B34" s="72" t="inlineStr">
+      <c r="B35" s="69" t="inlineStr">
         <is>
           <t>Competência x caixa — DECIDIR O REGIME</t>
         </is>
       </c>
-      <c r="C34" s="72" t="inlineStr">
+      <c r="C35" s="69" t="inlineStr">
         <is>
           <t>Confirmado pela gestora: TODOS os PJs das duas áreas prestam o serviço e recebem no mês seguinte — no Jurídico, Miguel, Thamar e Dra. Michele; no TI, Elias e Jonathan. O que foi pago em jan/26 é serviço de dez/2025, e o serviço de dez/26 só será pago em jan/2027. Hoje o realizado está lançado por CAIXA (mês do pagamento), que é como os valores foram informados, enquanto o orçamento foi montado por COMPETÊNCIA (mês do serviço). São bases diferentes no mesmo comparativo.</t>
         </is>
       </c>
-      <c r="D34" s="72" t="inlineStr">
+      <c r="D35" s="69" t="inlineStr">
         <is>
           <t>RECOMENDAÇÃO: migrar para competência, deslocando os PJs um mês para trás. Motivos: (1) o orçamento já é de competência, então acaba a comparação de bases diferentes; (2) por caixa, o ano de 2026 carrega um mês de 2025 e perde dez/26, o que distorce sempre que o valor muda no meio do ano — no Miguel, R$ 47.250 por caixa contra R$ 49.318 por competência em jan–jul, R$ 2.068 de diferença; (3) o SIENGE gera os dois regimes, então é escolha de configuração. Contra: caixa é mais fácil de bater com o extrato bancário. Decidir UMA vez e manter, senão o histórico mistura critérios. ATENÇÃO NO JONATHAN: o planejado dele começa em abr/26 (competência) e o realizado também foi lançado a partir de abr (caixa) — se ele recebe no mês seguinte, o pagamento de abril é serviço de março, e ou a entrada dele foi em março, ou o realizado de abril deveria ser zero. Conferir junto com a decisão do regime.</t>
         </is>
       </c>
-      <c r="E34" s="72" t="inlineStr">
+      <c r="E35" s="69" t="inlineStr">
         <is>
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F34" s="76" t="inlineStr">
+      <c r="F35" s="76" t="inlineStr">
         <is>
           <t>DECIDIR</t>
         </is>

</xml_diff>

<commit_message>
docs(orcamento): Office 365 — estrutura esclarecida, valor a confirmar
Gestora esclareceu que cada licenca atende 6 funcionarios, entao 10
licencas fecham os 60 usuarios da ficha — os numeros nao eram
contraditorios.

Falta confirmar se os R$ 440 sao por licenca ou o total mensal. Se
total: R$ 5.280/ano, R$ 780 acima do orcado. Se por licenca:
R$ 52.800/ano, R$ 48.300 acima — sozinho maior que todas as despesas
orcadas do TI. Registrado tambem que nao ha lancamento de
Microsoft/Office no extrato de jan a jul, o que precisa ser explicado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -29479,17 +29479,17 @@
       </c>
       <c r="B34" s="72" t="inlineStr">
         <is>
-          <t>Office 365 — nº de licenças</t>
+          <t>Office 365 — CONFIRMAR se R$ 440 é por licença ou o total</t>
         </is>
       </c>
       <c r="C34" s="72" t="inlineStr">
         <is>
-          <t>A observação diz '10 licenças de software – 60 usuários'. Os dois números não fecham entre si.</t>
+          <t>A gestora esclareceu a estrutura: cada licença atende 6 funcionários e custa R$ 440. Com 10 licenças, fecham os 60 usuários da ficha. Falta confirmar UMA coisa: os R$ 440 são o valor de CADA licença ou o total pago por mês? Não há lançamento de Microsoft/Office no extrato de jan a jul, o que também precisa ser explicado — é custo mensal e deveria aparecer.</t>
         </is>
       </c>
       <c r="D34" s="72" t="inlineStr">
         <is>
-          <t>Afeta o valor orçado da linha e a projeção de crescimento.</t>
+          <t>A diferença entre as duas leituras é enorme. Se R$ 440 for o total: R$ 5.280/ano, R$ 780 acima dos R$ 4.500 orçados — ajuste pequeno. Se for por licença: 10 x R$ 440 = R$ 4.400/mês, R$ 52.800/ano, R$ 48.300 acima do orçado — sozinho maior que todas as despesas orçadas do TI, e o orçamento da área estaria comprometido. Confirmar antes da reunião.</t>
         </is>
       </c>
       <c r="E34" s="72" t="inlineStr">
@@ -29499,7 +29499,7 @@
       </c>
       <c r="F34" s="74" t="inlineStr">
         <is>
-          <t>EM ABERTO</t>
+          <t>CONFIRMAR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(orcamento): divisao de responsabilidades no acompanhamento do TI
Item Y: o recorrente fica com o analista (Vinicius, 173 h/mes a
R$ 31,25/h) — extracao do SIENGE, lancamento, controle de equipamentos,
saldo por area, conferencia de faturas. O consultor (Jonathan, 3 dias
por semana, 104 h/mes a R$ 60,58/h) fica so com entregas pontuais e
tecnicas: avaliar AnyDesk x Monitor Remoto, avaliar Claude x GPT e
automatizar a extracao do SIENGE. A gestao fica com negociacao, rateio
e apresentacao.

Criterio registrado: 104 h/mes e capacidade limitada e a hora do
consultor custa o dobro da do analista, entao consultor em rotina
administrativa e o recurso mais caro na tarefa mais barata. Se ele
aparecer na rotina mensal, e sinal de que algo deveria ter sido
automatizado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -28486,7 +28486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -29474,22 +29474,22 @@
     <row r="34" ht="58" customHeight="1">
       <c r="A34" s="71" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B34" s="72" t="inlineStr">
         <is>
-          <t>Office 365 — CONFIRMAR se R$ 440 é por licença ou o total</t>
+          <t>Divisão de responsabilidades no acompanhamento</t>
         </is>
       </c>
       <c r="C34" s="72" t="inlineStr">
         <is>
-          <t>A gestora esclareceu a estrutura: cada licença atende 6 funcionários e custa R$ 440. Com 10 licenças, fecham os 60 usuários da ficha. Falta confirmar UMA coisa: os R$ 440 são o valor de CADA licença ou o total pago por mês? Não há lançamento de Microsoft/Office no extrato de jan a jul, o que também precisa ser explicado — é custo mensal e deveria aparecer.</t>
+          <t>Definição de quem faz o quê no controle orçamentário do TI. Capacidades: Vinicius, analista, 173 h/mês a R$ 31,25/h de custo total; Jonathan, consultor/desenvolvedor, 3 dias por semana, 104 h/mês a R$ 60,58/h — o dobro. Cristiane na gestão.</t>
         </is>
       </c>
       <c r="D34" s="72" t="inlineStr">
         <is>
-          <t>A diferença entre as duas leituras é enorme. Se R$ 440 for o total: R$ 5.280/ano, R$ 780 acima dos R$ 4.500 orçados — ajuste pequeno. Se for por licença: 10 x R$ 440 = R$ 4.400/mês, R$ 52.800/ano, R$ 48.300 acima do orçado — sozinho maior que todas as despesas orçadas do TI, e o orçamento da área estaria comprometido. Confirmar antes da reunião.</t>
+          <t>VINICIUS (todo o recorrente): extração mensal do SIENGE e lançamento do realizado, controle de equipamentos (solicitações, empréstimos, troca 1x1), acompanhamento do saldo por área para avisar antes do estouro, conferência de faturas contra contrato. JONATHAN (pontual e técnico, nunca rotina): avaliar AnyDesk x Monitor Remoto, avaliar Claude x GPT e planos de equipe, e automatizar a extração do SIENGE — esta última é a que paga o custo dele, porque devolve tempo do analista todos os meses. CRISTIANE: negociação de contratos, rateio, o que entra e sai do orçamento, apresentação à diretoria. Critério: 104 h/mês é capacidade limitada, e cada hora do consultor em tarefa administrativa custa o dobro da mesma hora do analista. Se o Jonathan aparecer na rotina mensal, é sinal de que algo deveria ter sido automatizado.</t>
         </is>
       </c>
       <c r="E34" s="72" t="inlineStr">
@@ -29497,39 +29497,71 @@
           <t>Cristiane</t>
         </is>
       </c>
-      <c r="F34" s="74" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
+      <c r="F34" s="73" t="inlineStr">
+        <is>
+          <t>APLICADO</t>
         </is>
       </c>
     </row>
     <row r="35" ht="58" customHeight="1">
       <c r="A35" s="68" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B35" s="69" t="inlineStr">
+        <is>
+          <t>Office 365 — CONFIRMAR se R$ 440 é por licença ou o total</t>
+        </is>
+      </c>
+      <c r="C35" s="69" t="inlineStr">
+        <is>
+          <t>A gestora esclareceu a estrutura: cada licença atende 6 funcionários e custa R$ 440. Com 10 licenças, fecham os 60 usuários da ficha. Falta confirmar UMA coisa: os R$ 440 são o valor de CADA licença ou o total pago por mês? Não há lançamento de Microsoft/Office no extrato de jan a jul, o que também precisa ser explicado — é custo mensal e deveria aparecer.</t>
+        </is>
+      </c>
+      <c r="D35" s="69" t="inlineStr">
+        <is>
+          <t>A diferença entre as duas leituras é enorme. Se R$ 440 for o total: R$ 5.280/ano, R$ 780 acima dos R$ 4.500 orçados — ajuste pequeno. Se for por licença: 10 x R$ 440 = R$ 4.400/mês, R$ 52.800/ano, R$ 48.300 acima do orçado — sozinho maior que todas as despesas orçadas do TI, e o orçamento da área estaria comprometido. Confirmar antes da reunião.</t>
+        </is>
+      </c>
+      <c r="E35" s="69" t="inlineStr">
+        <is>
+          <t>Cristiane</t>
+        </is>
+      </c>
+      <c r="F35" s="74" t="inlineStr">
+        <is>
+          <t>CONFIRMAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="58" customHeight="1">
+      <c r="A36" s="71" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B35" s="69" t="inlineStr">
+      <c r="B36" s="72" t="inlineStr">
         <is>
           <t>Competência x caixa — DECIDIR O REGIME</t>
         </is>
       </c>
-      <c r="C35" s="69" t="inlineStr">
+      <c r="C36" s="72" t="inlineStr">
         <is>
           <t>Confirmado pela gestora: TODOS os PJs das duas áreas prestam o serviço e recebem no mês seguinte — no Jurídico, Miguel, Thamar e Dra. Michele; no TI, Elias e Jonathan. O que foi pago em jan/26 é serviço de dez/2025, e o serviço de dez/26 só será pago em jan/2027. Hoje o realizado está lançado por CAIXA (mês do pagamento), que é como os valores foram informados, enquanto o orçamento foi montado por COMPETÊNCIA (mês do serviço). São bases diferentes no mesmo comparativo.</t>
         </is>
       </c>
-      <c r="D35" s="69" t="inlineStr">
+      <c r="D36" s="72" t="inlineStr">
         <is>
           <t>RECOMENDAÇÃO: migrar para competência, deslocando os PJs um mês para trás. Motivos: (1) o orçamento já é de competência, então acaba a comparação de bases diferentes; (2) por caixa, o ano de 2026 carrega um mês de 2025 e perde dez/26, o que distorce sempre que o valor muda no meio do ano — no Miguel, R$ 47.250 por caixa contra R$ 49.318 por competência em jan–jul, R$ 2.068 de diferença; (3) o SIENGE gera os dois regimes, então é escolha de configuração. Contra: caixa é mais fácil de bater com o extrato bancário. Decidir UMA vez e manter, senão o histórico mistura critérios. ATENÇÃO NO JONATHAN: o planejado dele começa em abr/26 (competência) e o realizado também foi lançado a partir de abr (caixa) — se ele recebe no mês seguinte, o pagamento de abril é serviço de março, e ou a entrada dele foi em março, ou o realizado de abril deveria ser zero. Conferir junto com a decisão do regime.</t>
         </is>
       </c>
-      <c r="E35" s="69" t="inlineStr">
+      <c r="E36" s="72" t="inlineStr">
         <is>
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F35" s="76" t="inlineStr">
+      <c r="F36" s="76" t="inlineStr">
         <is>
           <t>DECIDIR</t>
         </is>

</xml_diff>

<commit_message>
docs(orcamento): AnyDesk ainda nao contratado
Gestora confirmou que a contratacao nao ocorreu. Realizado zerado de
jan a jul, para a linha nao aparecer como falta de lancamento, e a
pendencia V atualizada.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -28623,13 +28623,27 @@
         <f>Planejado!G31</f>
         <v/>
       </c>
-      <c r="H31" s="58" t="n"/>
-      <c r="I31" s="58" t="n"/>
-      <c r="J31" s="58" t="n"/>
-      <c r="K31" s="58" t="n"/>
-      <c r="L31" s="58" t="n"/>
-      <c r="M31" s="58" t="n"/>
-      <c r="N31" s="58" t="n"/>
+      <c r="H31" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="58" t="n">
+        <v>0</v>
+      </c>
       <c r="O31" s="58" t="n"/>
       <c r="P31" s="58" t="n"/>
       <c r="Q31" s="58" t="n"/>
@@ -28639,8 +28653,16 @@
         <f>SUM(H31:S31)</f>
         <v/>
       </c>
-      <c r="U31" s="59" t="n"/>
-      <c r="V31" s="59" t="n"/>
+      <c r="U31" s="59" t="inlineStr">
+        <is>
+          <t>Gestora, 05/08/26</t>
+        </is>
+      </c>
+      <c r="V31" s="59" t="inlineStr">
+        <is>
+          <t>Ainda não contratado — sem custo até jul/26</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="56">
@@ -30817,7 +30839,7 @@
       </c>
       <c r="D32" s="72" t="inlineStr">
         <is>
-          <t>Não há sobreposição com o 'Monitor Remoto' do extrato: aquele credor é o Jonathan (J H Alves), consultor, não um software de acesso remoto. O AnyDesk é contratação nova e sem substituto atual. Definir valor e mês para a linha entrar no orçamento — enquanto o planejado for zero, qualquer lançamento aparece como 'Não orçado'.</t>
+          <t>Ainda não contratado — realizado zerado até jul/26, e não falta de lançamento. Não há sobreposição com o 'Monitor Remoto' do extrato: aquele credor é o Jonathan (J H Alves), consultor, não um software de acesso remoto. É contratação nova, sem substituto atual. Definir valor e mês antes de assinar — enquanto o planejado for zero, qualquer lançamento aparece como 'Não orçado'.</t>
         </is>
       </c>
       <c r="E32" s="72" t="inlineStr">

</xml_diff>

<commit_message>
feat(orcamento): sala de reuniao — executar so o funcional
Decisao da gestora. Entram cameras, microfones e cadeiras; saem
cafeteira, copos, canetas e blocos personalizados, que sao consumo e
brinde e pertencem ao Administrativo.

Falta a quebra do valor entre os dois grupos para ajustar a linha, hoje
em R$ 2.800/mes. Registrado tambem que o funcional melhora a qualidade
da reuniao, nao a capacidade — se o problema de espaco levantado pela
gestora precisar de solucao, e projeto a parte.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -26163,12 +26163,12 @@
       </c>
       <c r="D24" s="48" t="inlineStr">
         <is>
-          <t>Projeto Melhoria de Infraestrutura - Sala de Reunião</t>
+          <t>Projeto Sala de Reunião — itens funcionais</t>
         </is>
       </c>
       <c r="E24" s="48" t="inlineStr">
         <is>
-          <t>Cadeiras, cafeteira, copos, canetas, blocos personalizados, câmeras, microfones etc.</t>
+          <t>Câmeras, microfones e cadeiras. DECIDIDO executar só o funcional; cafeteira, copos, canetas e blocos personalizados saem para o Administrativo. Valor a rever quando vier a quebra entre funcional e consumo</t>
         </is>
       </c>
       <c r="F24" s="47" t="inlineStr"/>
@@ -30669,27 +30669,27 @@
       </c>
       <c r="B27" s="69" t="inlineStr">
         <is>
-          <t>Sala de Reunião — EXECUTAR, PAUSAR OU REPENSAR?</t>
+          <t>Sala de Reunião — DECIDIDO: executar só o funcional</t>
         </is>
       </c>
       <c r="C27" s="69" t="inlineStr">
         <is>
-          <t>Projeto orçado em R$ 2.800/mês × 12 = R$ 33.600, classificado em Móveis e Utensílios, sem nenhum lançamento até jul/26. A gestora levanta que a sala já não comporta todas as pessoas, então investir na configuração atual pode não resolver o problema real. Três caminhos: executar como está, pausar, ou repensar a solução (outro espaço, formato híbrido, mais de uma sala).</t>
+          <t>DECISÃO DA GESTORA: mexer somente no que for funcional. Entram os itens de infraestrutura de reunião — câmeras, microfones e cadeiras. Ficam de fora cafeteira, copos, canetas e blocos personalizados, que são consumo e brinde, pertencem ao Administrativo (item U) e não resolvem o problema da sala. O orçamento atual é de R$ 2.800/mês, R$ 33.600 no ano, sem nenhum lançamento até jul/26.</t>
         </is>
       </c>
       <c r="D27" s="69" t="inlineStr">
         <is>
-          <t>É a maior despesa isolada do TI e 38% de tudo que a área tem orçado em despesas. Se pausar, são R$ 33.600 liberados — mais que a economia atual do departamento. Decidir antes de comprometer o valor. Se a decisão for executar, definir também se é compra pontual ou parcelada: hoje está diluída linearmente, e se for compra única o desvio mensal vai acusar economia falsa todo mês até a compra e um pico no mês em que ocorrer. SEPARAR OS ITENS: a descrição na ficha mistura infraestrutura de reunião (câmeras, microfones, cadeiras) com material de consumo e brindes (canetas, blocos personalizados, copos, cafeteira). O segundo grupo é papelaria e deveria estar no Administrativo, não no TI (item U).</t>
+          <t>FALTA A QUEBRA DO VALOR: quanto dos R$ 33.600 é funcional e quanto é consumo. Só com isso dá para ajustar a linha e liberar a diferença. Levantar orçamento dos itens funcionais antes de comprar. Definir também se é compra pontual ou parcelada — hoje está diluída linearmente em 12 meses, e se for compra única o desvio vai acusar economia falsa todo mês até a compra e um pico no mês em que ocorrer. Segue de pé a observação da gestora de que a sala já não comporta todas as pessoas: o funcional melhora a qualidade da reunião, não a capacidade — se o problema de espaço precisar de solução, é projeto à parte.</t>
         </is>
       </c>
       <c r="E27" s="69" t="inlineStr">
         <is>
-          <t>Cristiane + Diretoria</t>
-        </is>
-      </c>
-      <c r="F27" s="76" t="inlineStr">
-        <is>
-          <t>PAUTA REUNIÃO</t>
+          <t>Cristiane</t>
+        </is>
+      </c>
+      <c r="F27" s="74" t="inlineStr">
+        <is>
+          <t>QUEBRAR VALOR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(orcamento): politica de troca 1x1 aprovada, emprestimo de 7 dias
Gestora aprovou a regra e definiu o prazo: 7 dias corridos de
emprestimo, depois disso vira "Atrasado" e o TI cobra a devolucao.

A aba de Controle de Equipamentos ganhou a regra do prazo no bloco
inicial, o cabecalho da coluna passou a "Dias em posse (limite: 7)" e
uma formatacao condicional destaca em vermelho quem passar do prazo — o
calculo ja era automatico a partir da data de saida.

Pendencia T passa de IMPLANTAR para APROVADA. Restam tres
encaminhamentos: comunicar a regra as areas, montar o estoque reserva
com fio e verificar com o financeiro se o lancamento pode nascer no
centro de custo da area solicitante.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -24,7 +24,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparativo'!$A$5:$N$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Planejado'!$A$4:$T$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Controle de Equipamentos'!$A$11:$J$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Controle de Equipamentos'!$A$12:$J$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Contas Pagas (resumo)'!$A$4:$L$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Contas Pagas (detalhe)'!$A$4:$H$423</definedName>
   </definedNames>
@@ -2108,7 +2108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2187,12 +2187,12 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="90" t="inlineStr">
         <is>
-          <t>Sem devolução</t>
+          <t>Prazo: 7 dias</t>
         </is>
       </c>
       <c r="B7" s="85" t="inlineStr">
         <is>
-          <t>Se a pessoa não entrega o item antigo, a solicitação fica 'Pendente devolução' e não vira compra até ser resolvida.</t>
+          <t>O empréstimo vale por 7 dias corridos. Passou disso, o status vira 'Atrasado' e o TI cobra a devolução. A coluna 'Dias em posse' calcula sozinha a partir da data de saída.</t>
         </is>
       </c>
       <c r="C7" s="86" t="n"/>
@@ -2207,12 +2207,12 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="90" t="inlineStr">
         <is>
-          <t>Aviso de saldo</t>
+          <t>Sem devolução</t>
         </is>
       </c>
       <c r="B8" s="85" t="inlineStr">
         <is>
-          <t>Antes de aprovar, conferir o saldo da rubrica da área solicitante. Se a compra for levar ao estouro, avisar a área ANTES de comprar (pendência R).</t>
+          <t>Se a pessoa não entrega o item antigo, a solicitação fica 'Pendente devolução' e não vira compra até ser resolvida.</t>
         </is>
       </c>
       <c r="C8" s="86" t="n"/>
@@ -2224,76 +2224,84 @@
       <c r="I8" s="86" t="n"/>
       <c r="J8" s="86" t="n"/>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="83" t="inlineStr">
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="90" t="inlineStr">
+        <is>
+          <t>Aviso de saldo</t>
+        </is>
+      </c>
+      <c r="B9" s="85" t="inlineStr">
+        <is>
+          <t>Antes de aprovar, conferir o saldo da rubrica da área solicitante. Se a compra for levar ao estouro, avisar a área ANTES de comprar (pendência R).</t>
+        </is>
+      </c>
+      <c r="C9" s="86" t="n"/>
+      <c r="D9" s="86" t="n"/>
+      <c r="E9" s="86" t="n"/>
+      <c r="F9" s="86" t="n"/>
+      <c r="G9" s="86" t="n"/>
+      <c r="H9" s="86" t="n"/>
+      <c r="I9" s="86" t="n"/>
+      <c r="J9" s="86" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="83" t="inlineStr">
         <is>
           <t>SOLICITAÇÕES</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Área solicitante</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Solicitante</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Motivo</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Devolveu o antigo?</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>Patrimônio devolvido</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Valor estimado</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="91" t="n"/>
-      <c r="B12" s="91" t="n"/>
-      <c r="C12" s="91" t="n"/>
-      <c r="D12" s="91" t="n"/>
-      <c r="E12" s="91" t="n"/>
-      <c r="F12" s="91" t="n"/>
-      <c r="G12" s="91" t="n"/>
-      <c r="H12" s="58" t="n"/>
-      <c r="I12" s="91" t="n"/>
-      <c r="J12" s="91" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="91" t="n"/>
@@ -2763,79 +2771,76 @@
       <c r="I51" s="91" t="n"/>
       <c r="J51" s="91" t="n"/>
     </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="29" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="91" t="n"/>
+      <c r="B52" s="91" t="n"/>
+      <c r="C52" s="91" t="n"/>
+      <c r="D52" s="91" t="n"/>
+      <c r="E52" s="91" t="n"/>
+      <c r="F52" s="91" t="n"/>
+      <c r="G52" s="91" t="n"/>
+      <c r="H52" s="58" t="n"/>
+      <c r="I52" s="91" t="n"/>
+      <c r="J52" s="91" t="n"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="29" t="inlineStr">
         <is>
           <t>EMPRÉSTIMOS (equipamento reserva)</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="92" t="inlineStr">
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="92" t="inlineStr">
         <is>
           <t>Item emprestado</t>
         </is>
       </c>
-      <c r="B54" s="92" t="inlineStr">
+      <c r="B55" s="92" t="inlineStr">
         <is>
           <t>Patrimônio</t>
         </is>
       </c>
-      <c r="C54" s="92" t="inlineStr">
+      <c r="C55" s="92" t="inlineStr">
         <is>
           <t>Área</t>
         </is>
       </c>
-      <c r="D54" s="92" t="inlineStr">
+      <c r="D55" s="92" t="inlineStr">
         <is>
           <t>Pessoa</t>
         </is>
       </c>
-      <c r="E54" s="92" t="inlineStr">
+      <c r="E55" s="92" t="inlineStr">
         <is>
           <t>Saída em</t>
         </is>
       </c>
-      <c r="F54" s="92" t="inlineStr">
+      <c r="F55" s="92" t="inlineStr">
         <is>
           <t>Previsão de devolução</t>
         </is>
       </c>
-      <c r="G54" s="92" t="inlineStr">
+      <c r="G55" s="92" t="inlineStr">
         <is>
           <t>Devolvido em</t>
         </is>
       </c>
-      <c r="H54" s="92" t="inlineStr">
+      <c r="H55" s="92" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I54" s="92" t="inlineStr">
-        <is>
-          <t>Dias em posse</t>
-        </is>
-      </c>
-      <c r="J54" s="92" t="inlineStr">
+      <c r="I55" s="92" t="inlineStr">
+        <is>
+          <t>Dias em posse (limite: 7)</t>
+        </is>
+      </c>
+      <c r="J55" s="92" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="91" t="n"/>
-      <c r="B55" s="91" t="n"/>
-      <c r="C55" s="91" t="n"/>
-      <c r="D55" s="91" t="n"/>
-      <c r="E55" s="91" t="n"/>
-      <c r="F55" s="91" t="n"/>
-      <c r="G55" s="91" t="n"/>
-      <c r="H55" s="91" t="n"/>
-      <c r="I55" s="93">
-        <f>IF(E55="","",IF(G55="",TODAY()-E55,G55-E55))</f>
-        <v/>
-      </c>
-      <c r="J55" s="91" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="91" t="n"/>
@@ -3197,27 +3202,48 @@
       </c>
       <c r="J79" s="91" t="n"/>
     </row>
+    <row r="80">
+      <c r="A80" s="91" t="n"/>
+      <c r="B80" s="91" t="n"/>
+      <c r="C80" s="91" t="n"/>
+      <c r="D80" s="91" t="n"/>
+      <c r="E80" s="91" t="n"/>
+      <c r="F80" s="91" t="n"/>
+      <c r="G80" s="91" t="n"/>
+      <c r="H80" s="91" t="n"/>
+      <c r="I80" s="93">
+        <f>IF(E80="","",IF(G80="",TODAY()-E80,G80-E80))</f>
+        <v/>
+      </c>
+      <c r="J80" s="91" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A11:J51"/>
-  <mergeCells count="9">
+  <autoFilter ref="A12:J52"/>
+  <mergeCells count="10">
     <mergeCell ref="B7:J7"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="B5:J5"/>
-    <mergeCell ref="A53:J53"/>
+    <mergeCell ref="B9:J9"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="B8:J8"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A10:J10"/>
     <mergeCell ref="B6:J6"/>
+    <mergeCell ref="A54:J54"/>
+    <mergeCell ref="A11:J11"/>
   </mergeCells>
+  <conditionalFormatting sqref="I56:I80">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="I12:I51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I13:I52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Aberta,Aguardando devolução,Aprovada,Comprada,Entregue,Negada"</formula1>
     </dataValidation>
-    <dataValidation sqref="F12:F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F13:F52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não,Não se aplica"</formula1>
     </dataValidation>
-    <dataValidation sqref="H55:H79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H56:H80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Emprestado,Devolvido,Atrasado,Baixado"</formula1>
     </dataValidation>
   </dataValidations>
@@ -30775,17 +30801,17 @@
       </c>
       <c r="D30" s="72" t="inlineStr">
         <is>
-          <t>Além de controlar estoque, a troca 1x1 gera dado de durabilidade e padrão de uso — se uma área quebra três vezes mais que as outras, isso aparece. Encaminhar: (1) comunicar a regra às áreas; (2) montar o pequeno estoque de reserva; (3) definir quantos dias o empréstimo pode durar antes de virar 'Atrasado'; (4) verificar com o financeiro se o lançamento pode nascer no centro de custo da área solicitante — se puder, o controle de custo por área sai do próprio SIENGE e esta aba fica só para o que ainda não virou pagamento.</t>
+          <t>APROVADA pela gestora, com prazo de empréstimo de 7 DIAS CORRIDOS — passou disso, vira 'Atrasado' e o TI cobra a devolução. A aba de controle já destaca em vermelho quem passar do prazo. Além de controlar estoque, a troca 1x1 gera dado de durabilidade e padrão de uso: se uma área quebra três vezes mais que as outras, isso aparece. Falta encaminhar: (1) comunicar a regra e o prazo às áreas; (2) montar o estoque de reserva com fio; (3) verificar com o financeiro se o lançamento pode nascer no centro de custo da área solicitante — se puder, o controle de custo por área sai do próprio SIENGE e esta aba fica só para o que ainda não virou pagamento.</t>
         </is>
       </c>
       <c r="E30" s="72" t="inlineStr">
         <is>
-          <t>Cristiane</t>
+          <t>Cristiane + Vinicius</t>
         </is>
       </c>
       <c r="F30" s="74" t="inlineStr">
         <is>
-          <t>IMPLANTAR</t>
+          <t>APROVADA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(orcamento): papelaria confirmada no Administrativo
Gestora confirmou a direcao. Fica a verificar se ha papelaria caindo
hoje no orcamento ou no centro de custo do TI por motivo historico —
nesse caso entra no mesmo pedido de reclassificacao do Adapta. Os itens
de consumo do projeto da sala de reuniao (cafeteira, copos, canetas,
blocos personalizados) saem do TI por esta decisao.

Pendencia U passa de RECOMENDACAO para CONFIRMADA.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -30833,7 +30833,7 @@
       </c>
       <c r="D31" s="69" t="inlineStr">
         <is>
-          <t>Três diferenças separam as duas coisas: (1) papelaria acaba, não quebra, então a regra de troca 1x1 não se aplica — o controle é de estoque por ponto de pedido, outra lógica; (2) não há patrimônio nem número de série para rastrear item a item; (3) o custo de controlar uma caneta é maior que a caneta. Se papelaria estiver caindo no orçamento do TI por motivo histórico, é o mesmo caso do Adapta (item Q): classificação errada, corrigir na origem quando o centro de custo novo for aberto.</t>
+          <t>CONFIRMADO pela gestora: papelaria fica no Administrativo. Três diferenças sustentam a separação: (1) papelaria acaba, não quebra, então a regra de troca 1x1 não se aplica — o controle é de estoque por ponto de pedido, outra lógica; (2) não há patrimônio nem número de série para rastrear item a item; (3) o custo de controlar uma caneta é maior que a caneta. A VERIFICAR: se hoje há papelaria caindo no orçamento ou no centro de custo do TI por motivo histórico. Se houver, entra no mesmo pedido de reclassificação do Adapta (item Q). Vale conferir também os itens de consumo que estavam no projeto da sala de reunião — cafeteira, copos, canetas e blocos personalizados —, que por esta decisão saem do TI.</t>
         </is>
       </c>
       <c r="E31" s="69" t="inlineStr">
@@ -30843,7 +30843,7 @@
       </c>
       <c r="F31" s="74" t="inlineStr">
         <is>
-          <t>RECOMENDAÇÃO</t>
+          <t>CONFIRMADA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(orcamento): sala de reuniao aprovada no escopo completo
Gestora revisou a decisao: executar como esta, no escopo original, com
os itens de infraestrutura e os de consumo e ambientacao. Orcamento
mantido em R$ 2.800/mes, R$ 33.600 no ano. Revoga a decisao anterior de
executar so o funcional.

Item U ganhou a excecao correspondente: os itens de consumo deste
projeto ficam no TI por integrarem um projeto de ambientacao aprovado,
e nao por serem reposicao de material de escritorio.

Segue em aberto se e compra pontual ou parcelada — hoje diluida
linearmente em 12 meses, o que geraria economia falsa todo mes e um
pico no mes da compra se for aquisicao unica.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
+++ b/orcamento/Orcamento_Planejado_x_Realizado_2026.xlsx
@@ -26189,12 +26189,12 @@
       </c>
       <c r="D24" s="48" t="inlineStr">
         <is>
-          <t>Projeto Sala de Reunião — itens funcionais</t>
+          <t>Projeto Melhoria de Infraestrutura - Sala de Reunião</t>
         </is>
       </c>
       <c r="E24" s="48" t="inlineStr">
         <is>
-          <t>Câmeras, microfones e cadeiras. DECIDIDO executar só o funcional; cafeteira, copos, canetas e blocos personalizados saem para o Administrativo. Valor a rever quando vier a quebra entre funcional e consumo</t>
+          <t>Cadeiras, cafeteira, copos, canetas, blocos personalizados, câmeras, microfones etc. APROVADO no escopo completo. Definir se é compra pontual ou parcelada — hoje está diluída linearmente em 12 meses</t>
         </is>
       </c>
       <c r="F24" s="47" t="inlineStr"/>
@@ -30673,17 +30673,17 @@
       </c>
       <c r="B27" s="69" t="inlineStr">
         <is>
-          <t>Sala de Reunião — DECIDIDO: executar só o funcional</t>
+          <t>Sala de Reunião — DECIDIDO: executar o projeto completo</t>
         </is>
       </c>
       <c r="C27" s="69" t="inlineStr">
         <is>
-          <t>DECISÃO DA GESTORA: mexer somente no que for funcional. Entram os itens de infraestrutura de reunião — câmeras, microfones e cadeiras. Ficam de fora cafeteira, copos, canetas e blocos personalizados, que são consumo e brinde, pertencem ao Administrativo (item U) e não resolvem o problema da sala. O orçamento atual é de R$ 2.800/mês, R$ 33.600 no ano, sem nenhum lançamento até jul/26.</t>
+          <t>DECISÃO DA GESTORA: executar como está, no escopo original. Entram tanto os itens de infraestrutura (câmeras, microfones, cadeiras) quanto os de consumo e ambientação (cafeteira, copos, canetas e blocos personalizados). Orçamento mantido em R$ 2.800/mês, R$ 33.600 no ano, sem nenhum lançamento até jun/26. Revoga a decisão anterior de executar só o funcional.</t>
         </is>
       </c>
       <c r="D27" s="69" t="inlineStr">
         <is>
-          <t>FALTA A QUEBRA DO VALOR: quanto dos R$ 33.600 é funcional e quanto é consumo. Só com isso dá para ajustar a linha e liberar a diferença. Levantar orçamento dos itens funcionais antes de comprar. Definir também se é compra pontual ou parcelada — hoje está diluída linearmente em 12 meses, e se for compra única o desvio vai acusar economia falsa todo mês até a compra e um pico no mês em que ocorrer. Segue de pé a observação da gestora de que a sala já não comporta todas as pessoas: o funcional melhora a qualidade da reunião, não a capacidade — se o problema de espaço precisar de solução, é projeto à parte.</t>
+          <t>É a maior despesa isolada do TI e 38% do que a área tem orçado em despesas, então o mês em que a compra ocorrer vai dominar o comparativo. DEFINIR: se é compra pontual ou parcelada. Hoje está diluída linearmente em 12 meses — se for compra única, o desvio vai acusar economia falsa todo mês até a compra e um pico no mês em que ela acontecer; nesse caso vale concentrar o planejado no mês previsto. OBSERVAR: os itens de consumo e brinde deste projeto são a exceção à decisão do item U, que tirou papelaria do TI — aqui ficam por serem parte de um projeto de ambientação, não reposição de material de escritório. E a ressalva da própria gestora continua de pé: o projeto melhora a qualidade da reunião, não a capacidade da sala. Se o espaço não comporta todas as pessoas, isso segue verdade depois da compra.</t>
         </is>
       </c>
       <c r="E27" s="69" t="inlineStr">
@@ -30693,7 +30693,7 @@
       </c>
       <c r="F27" s="74" t="inlineStr">
         <is>
-          <t>QUEBRAR VALOR</t>
+          <t>APROVADO</t>
         </is>
       </c>
     </row>

</xml_diff>